<commit_message>
fix: corrige Excel y responsables MIPER
</commit_message>
<xml_diff>
--- a/docs/evidencias-ds44-miper/MIPER-NEXTPREV-MIPER-PRUEBA-001-V1.xlsx
+++ b/docs/evidencias-ds44-miper/MIPER-NEXTPREV-MIPER-PRUEBA-001-V1.xlsx
@@ -11,7 +11,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">MIPER!$11:$13</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">MIPER!$A$1:$P$27</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">MIPER!$A$1:$P$20</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -664,7 +664,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P27"/>
+  <dimension ref="A1:P20"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -839,7 +839,7 @@
         <v>Código</v>
       </c>
       <c r="B4" t="str" s="5">
-        <v>MIPER-PRUEBA-001</v>
+        <v>MIPER-001</v>
       </c>
       <c r="C4" t="str" s="5">
         <v/>
@@ -851,7 +851,7 @@
         <v>Versión</v>
       </c>
       <c r="F4" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G4" t="str" s="5">
         <v/>
@@ -889,7 +889,7 @@
         <v>Entidad empleadora</v>
       </c>
       <c r="B5" t="str" s="5">
-        <v>Empresa demostrativa NextPrev</v>
+        <v>Empresa Demo</v>
       </c>
       <c r="C5" t="str" s="5">
         <v/>
@@ -913,7 +913,7 @@
         <v>Centro de trabajo</v>
       </c>
       <c r="J5" t="str" s="5">
-        <v>Casa matriz / Principal</v>
+        <v>Centro Norte</v>
       </c>
       <c r="K5" t="str" s="5">
         <v/>
@@ -939,7 +939,7 @@
         <v>Proceso</v>
       </c>
       <c r="B6" t="str" s="5">
-        <v>Recepción, almacenamiento y despacho</v>
+        <v>Operacion mina</v>
       </c>
       <c r="C6" t="str" s="5">
         <v/>
@@ -963,7 +963,7 @@
         <v>Responsable proceso</v>
       </c>
       <c r="J6" t="str" s="5">
-        <v>Jefatura de operaciones</v>
+        <v>Camila Soto</v>
       </c>
       <c r="K6" t="str" s="5">
         <v/>
@@ -1086,43 +1086,43 @@
     </row>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B9" t="str" s="7">
         <v/>
       </c>
       <c r="C9" s="7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D9" t="str" s="7">
         <v/>
       </c>
       <c r="E9" s="7">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F9" t="str" s="7">
         <v/>
       </c>
       <c r="G9" s="7">
+        <v>0</v>
+      </c>
+      <c r="H9" t="str" s="7">
+        <v/>
+      </c>
+      <c r="I9" s="7">
         <v>1</v>
       </c>
-      <c r="H9" t="str" s="7">
-        <v/>
-      </c>
-      <c r="I9" s="7">
-        <v>7</v>
-      </c>
       <c r="J9" t="str" s="7">
         <v/>
       </c>
       <c r="K9" s="7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L9" t="str" s="7">
         <v/>
       </c>
       <c r="M9" s="7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N9" t="str" s="7">
         <v/>
@@ -1336,31 +1336,33 @@
     </row>
     <row r="14" xml:space="preserve">
       <c r="A14" t="str" s="11">
-        <v>Recepción, almacenamiento y despacho</v>
+        <v>Operacion mina</v>
       </c>
       <c r="B14" t="str" s="11">
-        <v>Operador de bodega</v>
+        <v>Operador</v>
       </c>
       <c r="C14" t="str" s="11">
-        <v>Recepcionar y almacenar materiales</v>
+        <v>Traslado interno</v>
       </c>
       <c r="D14" t="str" s="11">
-        <v>Gente: Personas expuestas durante la tarea | Equipos: Equipos móviles y herramientas | Materiales: Materiales almacenados | Ambiente: Superficie y condiciones del lugar | Detalle: Interacción observable durante la ejecución</v>
+        <v>Gente: Conductor fatigado | Equipos: Camioneta en maniobra | Detalle: Cruce sin demarcacion</v>
       </c>
       <c r="E14" t="str" s="11">
-        <v>Caídas al mismo nivel (A1)</v>
-      </c>
-      <c r="F14" t="str" s="11">
-        <v/>
-      </c>
-      <c r="G14" t="str" s="11">
-        <v/>
-      </c>
-      <c r="H14" t="str" s="11">
-        <v/>
-      </c>
-      <c r="I14" t="str" s="13">
-        <v/>
+        <v>Atropello (I1)</v>
+      </c>
+      <c r="F14" s="11">
+        <v>2</v>
+      </c>
+      <c r="G14" s="11">
+        <v>2</v>
+      </c>
+      <c r="H14" s="11">
+        <f>F14*G14</f>
+        <v>4</v>
+      </c>
+      <c r="I14" t="str" s="11">
+        <f>IF(H14&lt;=2,"Tolerable",IF(H14=4,"Moderado",IF(H14=8,"Importante","Intolerable")))</f>
+        <v>Moderado</v>
       </c>
       <c r="J14" t="str" s="11">
         <v/>
@@ -1381,597 +1383,214 @@
         <v/>
       </c>
       <c r="P14" t="str" xml:space="preserve" s="11">
-        <v xml:space="preserve">Administrativo: Demarcar rutas y verificar orden y limpieza
-Responsable: Jefatura de operaciones
-Plazo: 2026-08-15
+        <v xml:space="preserve">Administrativo: Control de velocidad
+Responsable: Juan Soto
+Plazo: 2026-07-20
 Estado: pendiente</v>
       </c>
     </row>
-    <row r="15" xml:space="preserve">
-      <c r="A15" t="str" s="12">
-        <v>Recepción, almacenamiento y despacho</v>
-      </c>
-      <c r="B15" t="str" s="12">
-        <v>Operador de bodega</v>
-      </c>
-      <c r="C15" t="str" s="12">
-        <v>Recepcionar y almacenar materiales</v>
-      </c>
-      <c r="D15" t="str" s="12">
-        <v>Gente: Personas expuestas durante la tarea | Equipos: Equipos móviles y herramientas | Materiales: Materiales almacenados | Ambiente: Superficie y condiciones del lugar | Detalle: Interacción observable durante la ejecución</v>
-      </c>
-      <c r="E15" t="str" s="12">
-        <v>Caídas al mismo nivel (A1)</v>
-      </c>
-      <c r="F15" s="12">
-        <v>1</v>
-      </c>
-      <c r="G15" s="12">
-        <v>2</v>
-      </c>
-      <c r="H15" s="12">
-        <f>F15*G15</f>
-        <v>2</v>
-      </c>
-      <c r="I15" t="str" s="12">
-        <f>IF(H15&lt;=2,"Tolerable",IF(H15=4,"Moderado",IF(H15=8,"Importante","Intolerable")))</f>
-        <v>Tolerable</v>
-      </c>
-      <c r="J15" t="str" s="12">
-        <v/>
-      </c>
-      <c r="K15" t="str" s="12">
-        <v/>
-      </c>
-      <c r="L15" t="str" s="12">
-        <v/>
-      </c>
-      <c r="M15" t="str" s="12">
-        <v/>
-      </c>
-      <c r="N15" t="str" s="12">
-        <v/>
-      </c>
-      <c r="O15" t="str" s="12">
-        <v/>
-      </c>
-      <c r="P15" t="str" xml:space="preserve" s="12">
-        <v xml:space="preserve">Administrativo: Inspección diaria de superficies
-Responsable: Jefatura de operaciones
-Plazo: 2026-08-15
-Estado: implementado</v>
-      </c>
-    </row>
-    <row r="16" xml:space="preserve">
-      <c r="A16" t="str" s="29">
-        <v>Recepción, almacenamiento y despacho</v>
-      </c>
-      <c r="B16" t="str" s="29">
-        <v>Operador de bodega</v>
-      </c>
-      <c r="C16" t="str" s="29">
-        <v>Preparar pedidos para despacho</v>
-      </c>
-      <c r="D16" t="str" s="29">
-        <v>Gente: Personas expuestas durante la tarea | Equipos: Equipos móviles y herramientas | Materiales: Materiales almacenados | Ambiente: Superficie y condiciones del lugar | Detalle: Interacción observable durante la ejecución</v>
-      </c>
-      <c r="E16" t="str" s="29">
-        <v>Cortes por herramientas (B3)</v>
-      </c>
-      <c r="F16" s="29">
-        <v>2</v>
-      </c>
-      <c r="G16" s="29">
-        <v>2</v>
-      </c>
-      <c r="H16" s="29">
-        <f>F16*G16</f>
-        <v>4</v>
-      </c>
-      <c r="I16" t="str" s="29">
-        <f>IF(H16&lt;=2,"Tolerable",IF(H16=4,"Moderado",IF(H16=8,"Importante","Intolerable")))</f>
-        <v>Moderado</v>
-      </c>
-      <c r="J16" t="str" s="29">
-        <v/>
-      </c>
-      <c r="K16" t="str" s="29">
-        <v/>
-      </c>
-      <c r="L16" t="str" s="29">
-        <v/>
-      </c>
-      <c r="M16" t="str" s="29">
-        <v/>
-      </c>
-      <c r="N16" t="str" s="29">
-        <v/>
-      </c>
-      <c r="O16" t="str" s="29">
-        <v/>
-      </c>
-      <c r="P16" t="str" xml:space="preserve" s="29">
-        <v xml:space="preserve">Administrativo: Usar cuchillos de seguridad y capacitar al personal
-Responsable: Jefatura de operaciones
-Plazo: 2026-08-15
-Estado: pendiente</v>
-      </c>
-    </row>
-    <row r="17" xml:space="preserve">
-      <c r="A17" t="str" s="12">
-        <v>Recepción, almacenamiento y despacho</v>
-      </c>
-      <c r="B17" t="str" s="12">
-        <v>Operador de bodega</v>
-      </c>
-      <c r="C17" t="str" s="12">
-        <v>Preparar pedidos para despacho</v>
-      </c>
-      <c r="D17" t="str" s="12">
-        <v>Gente: Personas expuestas durante la tarea | Equipos: Equipos móviles y herramientas | Materiales: Materiales almacenados | Ambiente: Superficie y condiciones del lugar | Detalle: Interacción observable durante la ejecución</v>
-      </c>
-      <c r="E17" t="str" s="12">
-        <v>Caída de objetos (B2)</v>
-      </c>
-      <c r="F17" s="12">
-        <v>2</v>
-      </c>
-      <c r="G17" s="12">
-        <v>4</v>
-      </c>
-      <c r="H17" s="12">
-        <f>F17*G17</f>
-        <v>8</v>
-      </c>
-      <c r="I17" t="str" s="12">
-        <f>IF(H17&lt;=2,"Tolerable",IF(H17=4,"Moderado",IF(H17=8,"Importante","Intolerable")))</f>
-        <v>Importante</v>
-      </c>
-      <c r="J17" t="str" s="12">
-        <v/>
-      </c>
-      <c r="K17" t="str" s="12">
-        <v/>
-      </c>
-      <c r="L17" t="str" s="12">
-        <v/>
-      </c>
-      <c r="M17" t="str" s="12">
-        <v/>
-      </c>
-      <c r="N17" t="str" s="12">
-        <v/>
-      </c>
-      <c r="O17" t="str" s="12">
-        <v/>
-      </c>
-      <c r="P17" t="str" xml:space="preserve" s="12">
-        <v xml:space="preserve">Administrativo: Reorganizar almacenamiento pesado
-Responsable: Jefatura de operaciones
-Plazo: 2026-08-15
-Estado: en_revision
-Administrativo: Instalar topes de retención
-Responsable: Jefatura de operaciones
-Plazo: 2026-08-15
-Estado: pendiente</v>
-      </c>
-    </row>
-    <row r="18" xml:space="preserve">
-      <c r="A18" t="str" s="29">
-        <v>Recepción, almacenamiento y despacho</v>
-      </c>
-      <c r="B18" t="str" s="29">
-        <v>Supervisor de operaciones</v>
-      </c>
-      <c r="C18" t="str" s="29">
-        <v>Gestionar contingencias operacionales</v>
-      </c>
-      <c r="D18" t="str" s="29">
-        <v>Gente: Personas expuestas durante la tarea | Equipos: Equipos móviles y herramientas | Materiales: Materiales almacenados | Ambiente: Superficie y condiciones del lugar | Detalle: Interacción observable durante la ejecución</v>
-      </c>
-      <c r="E18" t="str" s="29">
-        <v>Contacto eléctrico directo (F1)</v>
-      </c>
-      <c r="F18" s="29">
-        <v>4</v>
-      </c>
-      <c r="G18" s="29">
-        <v>4</v>
-      </c>
-      <c r="H18" s="29">
-        <f>F18*G18</f>
-        <v>16</v>
-      </c>
-      <c r="I18" t="str" s="29">
-        <f>IF(H18&lt;=2,"Tolerable",IF(H18=4,"Moderado",IF(H18=8,"Importante","Intolerable")))</f>
-        <v>Intolerable</v>
-      </c>
-      <c r="J18" t="str" s="29">
-        <v/>
-      </c>
-      <c r="K18" t="str" s="29">
-        <v/>
-      </c>
-      <c r="L18" t="str" s="29">
-        <v/>
-      </c>
-      <c r="M18" t="str" s="29">
-        <v/>
-      </c>
-      <c r="N18" t="str" s="29">
-        <v/>
-      </c>
-      <c r="O18" t="str" s="29">
-        <v/>
-      </c>
-      <c r="P18" t="str" xml:space="preserve" s="29">
-        <v xml:space="preserve">Administrativo: Retirar equipo defectuoso y bloquear energías
-Responsable: Jefatura de operaciones
-Plazo: 2026-08-15
-Estado: pendiente</v>
-      </c>
-    </row>
-    <row r="19" xml:space="preserve">
-      <c r="A19" t="str" s="30">
-        <v>Recepción, almacenamiento y despacho</v>
-      </c>
-      <c r="B19" t="str" s="30">
-        <v>Operador de bodega</v>
-      </c>
-      <c r="C19" t="str" s="30">
-        <v>Preparar pedidos para despacho</v>
-      </c>
-      <c r="D19" t="str" s="30">
-        <v>Gente: Personas expuestas durante la tarea | Equipos: Equipos móviles y herramientas | Materiales: Materiales almacenados | Ambiente: Superficie y condiciones del lugar | Detalle: Interacción observable durante la ejecución</v>
-      </c>
-      <c r="E19" t="str" s="30">
-        <v>Exposición a ruido (P1)</v>
-      </c>
-      <c r="F19" t="str" s="30">
-        <v/>
-      </c>
-      <c r="G19" t="str" s="30">
-        <v/>
-      </c>
-      <c r="H19" t="str" s="30">
-        <v/>
-      </c>
-      <c r="I19" t="str" s="30">
-        <v/>
-      </c>
-      <c r="J19" t="str" s="30">
-        <v>83 dB(A)</v>
-      </c>
-      <c r="K19" t="str" s="30">
-        <v>Sobre criterio de acción</v>
-      </c>
-      <c r="L19" t="str" s="30">
-        <v/>
-      </c>
-      <c r="M19" t="str" s="30">
-        <v/>
-      </c>
-      <c r="N19" t="str" s="30">
-        <v/>
-      </c>
-      <c r="O19" t="str" s="30">
-        <v/>
-      </c>
-      <c r="P19" t="str" xml:space="preserve" s="30">
-        <v xml:space="preserve">Administrativo: Implementar programa de conservación auditiva
-Responsable: Jefatura de operaciones
-Plazo: 2026-08-15
-Estado: pendiente</v>
-      </c>
-    </row>
-    <row r="20" xml:space="preserve">
-      <c r="A20" t="str" s="29">
-        <v>Recepción, almacenamiento y despacho</v>
-      </c>
-      <c r="B20" t="str" s="29">
-        <v>Supervisor de operaciones</v>
-      </c>
-      <c r="C20" t="str" s="29">
-        <v>Supervisar operación y coordinar turnos</v>
-      </c>
-      <c r="D20" t="str" s="29">
-        <v>Gente: Personas expuestas durante la tarea | Equipos: Equipos móviles y herramientas | Materiales: Materiales almacenados | Ambiente: Superficie y condiciones del lugar | Detalle: Interacción observable durante la ejecución</v>
-      </c>
-      <c r="E20" t="str" s="29">
-        <v>Carga de trabajo (D1)</v>
-      </c>
-      <c r="F20" t="str" s="29">
-        <v/>
-      </c>
-      <c r="G20" t="str" s="29">
-        <v/>
-      </c>
-      <c r="H20" t="str" s="29">
-        <v/>
-      </c>
-      <c r="I20" t="str" s="29">
-        <v/>
-      </c>
-      <c r="J20" t="str" s="29">
-        <v/>
-      </c>
-      <c r="K20" t="str" s="29">
-        <v/>
-      </c>
-      <c r="L20" t="str" s="29">
-        <v>CEAL-SM/SUSESO</v>
-      </c>
-      <c r="M20" t="str" s="29">
-        <v>Riesgo medio</v>
-      </c>
-      <c r="N20" t="str" s="29">
-        <v/>
-      </c>
-      <c r="O20" t="str" s="29">
-        <v/>
-      </c>
-      <c r="P20" t="str" xml:space="preserve" s="29">
-        <v xml:space="preserve">Administrativo: Revisar distribución de carga y pausas
-Responsable: Jefatura de operaciones
-Plazo: 2026-08-15
-Estado: pendiente</v>
-      </c>
-    </row>
-    <row r="21" xml:space="preserve">
-      <c r="A21" t="str" s="30">
-        <v>Recepción, almacenamiento y despacho</v>
-      </c>
-      <c r="B21" t="str" s="30">
-        <v>Operador de bodega</v>
-      </c>
-      <c r="C21" t="str" s="30">
-        <v>Recepcionar y almacenar materiales</v>
-      </c>
-      <c r="D21" t="str" s="30">
-        <v>Gente: Personas expuestas durante la tarea | Equipos: Equipos móviles y herramientas | Materiales: Materiales almacenados | Ambiente: Superficie y condiciones del lugar | Detalle: Interacción observable durante la ejecución</v>
-      </c>
-      <c r="E21" t="str" s="30">
-        <v>Manipulación manual de cargas (R1)</v>
-      </c>
-      <c r="F21" t="str" s="30">
-        <v/>
-      </c>
-      <c r="G21" t="str" s="30">
-        <v/>
-      </c>
-      <c r="H21" t="str" s="30">
-        <v/>
-      </c>
-      <c r="I21" t="str" s="30">
-        <v/>
-      </c>
-      <c r="J21" t="str" s="30">
-        <v/>
-      </c>
-      <c r="K21" t="str" s="30">
-        <v/>
-      </c>
-      <c r="L21" t="str" s="30">
-        <v/>
-      </c>
-      <c r="M21" t="str" s="30">
-        <v/>
-      </c>
-      <c r="N21" t="str" s="30">
-        <v>MAC nivel 3</v>
-      </c>
-      <c r="O21" t="str" s="30">
-        <v>Alto</v>
-      </c>
-      <c r="P21" t="str" xml:space="preserve" s="30">
-        <v xml:space="preserve">Administrativo: Incorporar ayuda mecánica para cargas
-Responsable: Jefatura de operaciones
-Plazo: 2026-08-15
-Estado: pendiente</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str" s="19">
+    <row r="16">
+      <c r="A16" t="str" s="19">
         <v>Firmas y aprobación</v>
       </c>
-      <c r="B23" t="str" s="19">
-        <v/>
-      </c>
-      <c r="C23" t="str" s="19">
-        <v/>
-      </c>
-      <c r="D23" t="str" s="19">
-        <v/>
-      </c>
-      <c r="E23" t="str" s="19">
-        <v/>
-      </c>
-      <c r="F23" t="str" s="19">
-        <v/>
-      </c>
-      <c r="G23" t="str" s="19">
-        <v/>
-      </c>
-      <c r="H23" t="str" s="19">
-        <v/>
-      </c>
-      <c r="I23" t="str" s="19">
-        <v/>
-      </c>
-      <c r="J23" t="str" s="19">
-        <v/>
-      </c>
-      <c r="K23" t="str" s="19">
-        <v/>
-      </c>
-      <c r="L23" t="str" s="19">
-        <v/>
-      </c>
-      <c r="M23" t="str" s="19">
-        <v/>
-      </c>
-      <c r="N23" t="str" s="19">
-        <v/>
-      </c>
-      <c r="O23" t="str" s="19">
-        <v/>
-      </c>
-      <c r="P23" t="str" s="19">
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="str" s="20">
+      <c r="B16" t="str" s="19">
+        <v/>
+      </c>
+      <c r="C16" t="str" s="19">
+        <v/>
+      </c>
+      <c r="D16" t="str" s="19">
+        <v/>
+      </c>
+      <c r="E16" t="str" s="19">
+        <v/>
+      </c>
+      <c r="F16" t="str" s="19">
+        <v/>
+      </c>
+      <c r="G16" t="str" s="19">
+        <v/>
+      </c>
+      <c r="H16" t="str" s="19">
+        <v/>
+      </c>
+      <c r="I16" t="str" s="19">
+        <v/>
+      </c>
+      <c r="J16" t="str" s="19">
+        <v/>
+      </c>
+      <c r="K16" t="str" s="19">
+        <v/>
+      </c>
+      <c r="L16" t="str" s="19">
+        <v/>
+      </c>
+      <c r="M16" t="str" s="19">
+        <v/>
+      </c>
+      <c r="N16" t="str" s="19">
+        <v/>
+      </c>
+      <c r="O16" t="str" s="19">
+        <v/>
+      </c>
+      <c r="P16" t="str" s="19">
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str" s="20">
         <v>Elaborado por</v>
       </c>
-      <c r="B25" t="str" s="5">
-        <v>Diana Marín · Prevencionista de riesgos</v>
-      </c>
-      <c r="C25" t="str" s="5">
-        <v/>
-      </c>
-      <c r="D25" t="str" s="5">
-        <v/>
-      </c>
-      <c r="E25" t="str" s="5">
-        <v/>
-      </c>
-      <c r="F25" t="str" s="20">
+      <c r="B18" t="str" s="5">
+        <v>Ana Perez</v>
+      </c>
+      <c r="C18" t="str" s="5">
+        <v/>
+      </c>
+      <c r="D18" t="str" s="5">
+        <v/>
+      </c>
+      <c r="E18" t="str" s="5">
+        <v/>
+      </c>
+      <c r="F18" t="str" s="20">
         <v>Fecha</v>
       </c>
-      <c r="G25" t="str" s="5">
+      <c r="G18" t="str" s="5">
         <v>2026-07-20</v>
       </c>
-      <c r="H25" t="str" s="5">
-        <v/>
-      </c>
-      <c r="I25" t="str" s="20">
+      <c r="H18" t="str" s="5">
+        <v/>
+      </c>
+      <c r="I18" t="str" s="20">
         <v>Revisado por</v>
       </c>
-      <c r="J25" t="str" s="5">
+      <c r="J18" t="str" s="5">
         <v>No informado</v>
       </c>
-      <c r="K25" t="str" s="5">
-        <v/>
-      </c>
-      <c r="L25" t="str" s="5">
-        <v/>
-      </c>
-      <c r="M25" t="str" s="20">
+      <c r="K18" t="str" s="5">
+        <v/>
+      </c>
+      <c r="L18" t="str" s="5">
+        <v/>
+      </c>
+      <c r="M18" t="str" s="20">
         <v>Fecha</v>
       </c>
-      <c r="N25" t="str" s="5">
+      <c r="N18" t="str" s="5">
         <v>Pendiente</v>
       </c>
-      <c r="O25" t="str" s="5">
-        <v/>
-      </c>
-      <c r="P25" t="str" s="5">
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="str" s="20">
+      <c r="O18" t="str" s="5">
+        <v/>
+      </c>
+      <c r="P18" t="str" s="5">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str" s="20">
         <v>Cargo / rol</v>
       </c>
-      <c r="B26" t="str" s="5">
+      <c r="B19" t="str" s="5">
         <v>Prevención de riesgos</v>
       </c>
-      <c r="C26" t="str" s="5">
-        <v/>
-      </c>
-      <c r="D26" t="str" s="5">
-        <v/>
-      </c>
-      <c r="E26" t="str" s="5">
-        <v/>
-      </c>
-      <c r="F26" t="str" s="20">
-        <v/>
-      </c>
-      <c r="G26" t="str" s="5">
-        <v/>
-      </c>
-      <c r="H26" t="str" s="5">
-        <v/>
-      </c>
-      <c r="I26" t="str" s="20">
+      <c r="C19" t="str" s="5">
+        <v/>
+      </c>
+      <c r="D19" t="str" s="5">
+        <v/>
+      </c>
+      <c r="E19" t="str" s="5">
+        <v/>
+      </c>
+      <c r="F19" t="str" s="20">
+        <v/>
+      </c>
+      <c r="G19" t="str" s="5">
+        <v/>
+      </c>
+      <c r="H19" t="str" s="5">
+        <v/>
+      </c>
+      <c r="I19" t="str" s="20">
         <v>Cargo / rol</v>
       </c>
-      <c r="J26" t="str" s="5">
+      <c r="J19" t="str" s="5">
         <v>Pendiente</v>
       </c>
-      <c r="K26" t="str" s="5">
-        <v/>
-      </c>
-      <c r="L26" t="str" s="5">
-        <v/>
-      </c>
-      <c r="M26" t="str" s="20">
-        <v/>
-      </c>
-      <c r="N26" t="str" s="5">
-        <v/>
-      </c>
-      <c r="O26" t="str" s="5">
-        <v/>
-      </c>
-      <c r="P26" t="str" s="5">
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="str" s="20">
+      <c r="K19" t="str" s="5">
+        <v/>
+      </c>
+      <c r="L19" t="str" s="5">
+        <v/>
+      </c>
+      <c r="M19" t="str" s="20">
+        <v/>
+      </c>
+      <c r="N19" t="str" s="5">
+        <v/>
+      </c>
+      <c r="O19" t="str" s="5">
+        <v/>
+      </c>
+      <c r="P19" t="str" s="5">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str" s="20">
         <v>Aprobado por</v>
       </c>
-      <c r="B27" t="str" s="5">
+      <c r="B20" t="str" s="5">
         <v>No informado</v>
       </c>
-      <c r="C27" t="str" s="5">
-        <v/>
-      </c>
-      <c r="D27" t="str" s="5">
-        <v/>
-      </c>
-      <c r="E27" t="str" s="5">
-        <v/>
-      </c>
-      <c r="F27" t="str" s="20">
+      <c r="C20" t="str" s="5">
+        <v/>
+      </c>
+      <c r="D20" t="str" s="5">
+        <v/>
+      </c>
+      <c r="E20" t="str" s="5">
+        <v/>
+      </c>
+      <c r="F20" t="str" s="20">
         <v>Fecha</v>
       </c>
-      <c r="G27" t="str" s="5">
+      <c r="G20" t="str" s="5">
         <v>Pendiente</v>
       </c>
-      <c r="H27" t="str" s="5">
-        <v/>
-      </c>
-      <c r="I27" t="str" s="20">
+      <c r="H20" t="str" s="5">
+        <v/>
+      </c>
+      <c r="I20" t="str" s="20">
         <v>Cargo / rol</v>
       </c>
-      <c r="J27" t="str" s="5">
+      <c r="J20" t="str" s="5">
         <v>Pendiente</v>
       </c>
-      <c r="K27" t="str" s="5">
-        <v/>
-      </c>
-      <c r="L27" t="str" s="5">
-        <v/>
-      </c>
-      <c r="M27" t="str" s="20">
-        <v/>
-      </c>
-      <c r="N27" t="str" s="5">
-        <v/>
-      </c>
-      <c r="O27" t="str" s="5">
-        <v/>
-      </c>
-      <c r="P27" t="str" s="5">
+      <c r="K20" t="str" s="5">
+        <v/>
+      </c>
+      <c r="L20" t="str" s="5">
+        <v/>
+      </c>
+      <c r="M20" t="str" s="20">
+        <v/>
+      </c>
+      <c r="N20" t="str" s="5">
+        <v/>
+      </c>
+      <c r="O20" t="str" s="5">
+        <v/>
+      </c>
+      <c r="P20" t="str" s="5">
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A13:P21"/>
+  <autoFilter ref="A13:P14"/>
   <mergeCells count="50">
     <mergeCell ref="A1:C2"/>
     <mergeCell ref="D1:P2"/>
@@ -2010,119 +1629,116 @@
     <mergeCell ref="J12:K12"/>
     <mergeCell ref="L12:M12"/>
     <mergeCell ref="N12:O12"/>
-    <mergeCell ref="A23:P23"/>
-    <mergeCell ref="B25:E25"/>
-    <mergeCell ref="G25:H25"/>
-    <mergeCell ref="J25:L25"/>
-    <mergeCell ref="N25:P25"/>
-    <mergeCell ref="B26:E26"/>
-    <mergeCell ref="G26:H26"/>
-    <mergeCell ref="J26:L26"/>
-    <mergeCell ref="N26:P26"/>
-    <mergeCell ref="B27:E27"/>
-    <mergeCell ref="G27:H27"/>
-    <mergeCell ref="J27:L27"/>
-    <mergeCell ref="N27:P27"/>
+    <mergeCell ref="A16:P16"/>
+    <mergeCell ref="B18:E18"/>
+    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="J18:L18"/>
+    <mergeCell ref="N18:P18"/>
+    <mergeCell ref="B19:E19"/>
+    <mergeCell ref="G19:H19"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="N19:P19"/>
+    <mergeCell ref="B20:E20"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="J20:L20"/>
+    <mergeCell ref="N20:P20"/>
   </mergeCells>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P27"/>
-  </ignoredErrors>
-  <conditionalFormatting sqref="I14:I21">
+  <conditionalFormatting sqref="I14:I14">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>EXACT(I14,"Evaluación pendiente")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I14:I21">
+  <conditionalFormatting sqref="I14:I14">
     <cfRule type="expression" dxfId="1" priority="2">
       <formula>EXACT(I14,"Tolerable")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I14:I21">
+  <conditionalFormatting sqref="I14:I14">
     <cfRule type="expression" dxfId="2" priority="3">
       <formula>EXACT(I14,"Moderado")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I14:I21">
+  <conditionalFormatting sqref="I14:I14">
     <cfRule type="expression" dxfId="3" priority="4">
       <formula>EXACT(I14,"Importante")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I14:I21">
+  <conditionalFormatting sqref="I14:I14">
     <cfRule type="expression" dxfId="4" priority="5">
       <formula>EXACT(I14,"Intolerable")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K14:K21">
+  <conditionalFormatting sqref="K14:K14">
     <cfRule type="expression" dxfId="0" priority="6">
       <formula>EXACT(K14,"Evaluación pendiente")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K14:K21">
+  <conditionalFormatting sqref="K14:K14">
     <cfRule type="expression" dxfId="1" priority="7">
       <formula>EXACT(K14,"Tolerable")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K14:K21">
+  <conditionalFormatting sqref="K14:K14">
     <cfRule type="expression" dxfId="2" priority="8">
       <formula>EXACT(K14,"Moderado")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K14:K21">
+  <conditionalFormatting sqref="K14:K14">
     <cfRule type="expression" dxfId="3" priority="9">
       <formula>EXACT(K14,"Importante")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K14:K21">
+  <conditionalFormatting sqref="K14:K14">
     <cfRule type="expression" dxfId="4" priority="10">
       <formula>EXACT(K14,"Intolerable")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M14:M21">
+  <conditionalFormatting sqref="M14:M14">
     <cfRule type="expression" dxfId="0" priority="11">
       <formula>EXACT(M14,"Evaluación pendiente")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M14:M21">
+  <conditionalFormatting sqref="M14:M14">
     <cfRule type="expression" dxfId="1" priority="12">
       <formula>EXACT(M14,"Tolerable")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M14:M21">
+  <conditionalFormatting sqref="M14:M14">
     <cfRule type="expression" dxfId="2" priority="13">
       <formula>EXACT(M14,"Moderado")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M14:M21">
+  <conditionalFormatting sqref="M14:M14">
     <cfRule type="expression" dxfId="3" priority="14">
       <formula>EXACT(M14,"Importante")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M14:M21">
+  <conditionalFormatting sqref="M14:M14">
     <cfRule type="expression" dxfId="4" priority="15">
       <formula>EXACT(M14,"Intolerable")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O14:O21">
+  <conditionalFormatting sqref="O14:O14">
     <cfRule type="expression" dxfId="0" priority="16">
       <formula>EXACT(O14,"Evaluación pendiente")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O14:O21">
+  <conditionalFormatting sqref="O14:O14">
     <cfRule type="expression" dxfId="1" priority="17">
       <formula>EXACT(O14,"Tolerable")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O14:O21">
+  <conditionalFormatting sqref="O14:O14">
     <cfRule type="expression" dxfId="2" priority="18">
       <formula>EXACT(O14,"Moderado")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O14:O21">
+  <conditionalFormatting sqref="O14:O14">
     <cfRule type="expression" dxfId="3" priority="19">
       <formula>EXACT(O14,"Importante")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O14:O21">
+  <conditionalFormatting sqref="O14:O14">
     <cfRule type="expression" dxfId="4" priority="20">
       <formula>EXACT(O14,"Intolerable")</formula>
     </cfRule>
@@ -2131,14 +1747,14 @@
   <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.45" header="0.15" footer="0.2"/>
   <pageSetup paperSize="8" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
   <headerFooter>
-    <oddFooter>MIPER-PRUEBA-001 V1 | borrador | 2026-07-20 | Página &amp;P de &amp;N</oddFooter>
+    <oddFooter>MIPER-001 V3 | borrador | 2026-07-21 | Página &amp;P de &amp;N</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K3"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -2195,152 +1811,44 @@
     </row>
     <row r="3">
       <c r="A3" t="str" s="23">
-        <v>Recepción, almacenamiento y despacho</v>
+        <v>Operacion mina</v>
       </c>
       <c r="B3" t="str" s="23">
         <v>operacional</v>
       </c>
       <c r="C3" t="str" s="23">
-        <v>Operador de bodega</v>
+        <v>Operador</v>
       </c>
       <c r="D3" t="str" s="23">
-        <v>Recepcionar y almacenar materiales</v>
+        <v>Traslado interno</v>
       </c>
       <c r="E3" t="str" s="23">
         <v>Sí</v>
       </c>
       <c r="F3" t="str" s="23">
-        <v>Bodega central</v>
+        <v>Patio A</v>
       </c>
       <c r="G3" s="23">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H3" t="str" s="23">
-        <v>hombre: 2 | mujer: 2</v>
+        <v>hombre: 2 | mujer: 1</v>
       </c>
       <c r="I3" t="str" s="23">
-        <v>Gente: Personas expuestas durante la tarea | Equipos: Equipos móviles y herramientas | Materiales: Materiales almacenados | Ambiente: Superficie y condiciones del lugar | Detalle: Interacción observable durante la ejecución</v>
+        <v>Gente: Conductor fatigado | Equipos: Camioneta en maniobra | Detalle: Cruce sin demarcacion</v>
       </c>
       <c r="J3" t="str" s="23">
-        <v>A1 Caídas al mismo nivel | R1 Manipulación manual de cargas</v>
+        <v>I1 Atropello</v>
       </c>
       <c r="K3" t="str" s="23">
-        <v>Turno diurno</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str" s="24">
-        <v>Recepción, almacenamiento y despacho</v>
-      </c>
-      <c r="B4" t="str" s="24">
-        <v>operacional</v>
-      </c>
-      <c r="C4" t="str" s="24">
-        <v>Operador de bodega</v>
-      </c>
-      <c r="D4" t="str" s="24">
-        <v>Preparar pedidos para despacho</v>
-      </c>
-      <c r="E4" t="str" s="24">
-        <v>Sí</v>
-      </c>
-      <c r="F4" t="str" s="24">
-        <v>Zona de picking</v>
-      </c>
-      <c r="G4" s="24">
-        <v>3</v>
-      </c>
-      <c r="H4" t="str" s="24">
-        <v>hombre: 2 | mujer: 1</v>
-      </c>
-      <c r="I4" t="str" s="24">
-        <v>Gente: Personas expuestas durante la tarea | Equipos: Equipos móviles y herramientas | Materiales: Materiales almacenados | Ambiente: Superficie y condiciones del lugar | Detalle: Interacción observable durante la ejecución</v>
-      </c>
-      <c r="J4" t="str" s="24">
-        <v>B3 Cortes por herramientas | B2 Caída de objetos | P1 Exposición a ruido</v>
-      </c>
-      <c r="K4" t="str" s="24">
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str" s="23">
-        <v>Recepción, almacenamiento y despacho</v>
-      </c>
-      <c r="B5" t="str" s="23">
-        <v>operacional</v>
-      </c>
-      <c r="C5" t="str" s="23">
-        <v>Supervisor de operaciones</v>
-      </c>
-      <c r="D5" t="str" s="23">
-        <v>Supervisar operación y coordinar turnos</v>
-      </c>
-      <c r="E5" t="str" s="23">
-        <v>Sí</v>
-      </c>
-      <c r="F5" t="str" s="23">
-        <v>Bodega y oficina</v>
-      </c>
-      <c r="G5" s="23">
-        <v>2</v>
-      </c>
-      <c r="H5" t="str" s="23">
-        <v>hombre: 1 | mujer: 1</v>
-      </c>
-      <c r="I5" t="str" s="23">
-        <v>Gente: Personas expuestas durante la tarea | Equipos: Equipos móviles y herramientas | Materiales: Materiales almacenados | Ambiente: Superficie y condiciones del lugar | Detalle: Interacción observable durante la ejecución</v>
-      </c>
-      <c r="J5" t="str" s="23">
-        <v>D1 Carga de trabajo</v>
-      </c>
-      <c r="K5" t="str" s="23">
-        <v>Incluye recorridos</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str" s="24">
-        <v>Recepción, almacenamiento y despacho</v>
-      </c>
-      <c r="B6" t="str" s="24">
-        <v>operacional</v>
-      </c>
-      <c r="C6" t="str" s="24">
-        <v>Supervisor de operaciones</v>
-      </c>
-      <c r="D6" t="str" s="24">
-        <v>Gestionar contingencias operacionales</v>
-      </c>
-      <c r="E6" t="str" s="24">
-        <v>No</v>
-      </c>
-      <c r="F6" t="str" s="24">
-        <v>Instalación completa</v>
-      </c>
-      <c r="G6" s="24">
-        <v>2</v>
-      </c>
-      <c r="H6" t="str" s="24">
-        <v>hombre: 1 | mujer: 1</v>
-      </c>
-      <c r="I6" t="str" s="24">
-        <v>Gente: Personas expuestas durante la tarea | Equipos: Equipos móviles y herramientas | Materiales: Materiales almacenados | Ambiente: Superficie y condiciones del lugar | Detalle: Interacción observable durante la ejecución</v>
-      </c>
-      <c r="J6" t="str" s="24">
-        <v>F1 Contacto eléctrico directo</v>
-      </c>
-      <c r="K6" t="str" s="24">
-        <v>Según evento</v>
+        <v>Ruta principal</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:K6"/>
+  <autoFilter ref="A2:K3"/>
   <mergeCells count="1">
     <mergeCell ref="A1:K1"/>
   </mergeCells>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K6"/>
-  </ignoredErrors>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.45" header="0.15" footer="0.2"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
@@ -2352,7 +1860,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J3"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -2405,300 +1913,41 @@
     </row>
     <row r="3">
       <c r="A3" t="str" s="23">
-        <v>Recepción, almacenamiento y despacho</v>
+        <v>Operacion mina</v>
       </c>
       <c r="B3" t="str" s="23">
-        <v>Operador de bodega</v>
+        <v>Operador</v>
       </c>
       <c r="C3" t="str" s="23">
-        <v>Recepcionar y almacenar materiales</v>
+        <v>Traslado interno</v>
       </c>
       <c r="D3" t="str" s="23">
-        <v>A1</v>
+        <v>I1</v>
       </c>
       <c r="E3" t="str" s="23">
-        <v>Caídas al mismo nivel</v>
+        <v>Atropello</v>
       </c>
       <c r="F3" t="str" s="23">
         <v>Administrativo</v>
       </c>
       <c r="G3" t="str" s="23">
-        <v>Demarcar rutas y verificar orden y limpieza</v>
+        <v>Control de velocidad</v>
       </c>
       <c r="H3" t="str" s="23">
-        <v>Jefatura de operaciones</v>
+        <v>Juan Soto</v>
       </c>
       <c r="I3" t="str" s="23">
-        <v>2026-08-15</v>
+        <v>2026-07-20</v>
       </c>
       <c r="J3" t="str" s="25">
         <v>pendiente</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="str" s="24">
-        <v>Recepción, almacenamiento y despacho</v>
-      </c>
-      <c r="B4" t="str" s="24">
-        <v>Operador de bodega</v>
-      </c>
-      <c r="C4" t="str" s="24">
-        <v>Recepcionar y almacenar materiales</v>
-      </c>
-      <c r="D4" t="str" s="24">
-        <v>A1</v>
-      </c>
-      <c r="E4" t="str" s="24">
-        <v>Caídas al mismo nivel</v>
-      </c>
-      <c r="F4" t="str" s="24">
-        <v>Administrativo</v>
-      </c>
-      <c r="G4" t="str" s="24">
-        <v>Inspección diaria de superficies</v>
-      </c>
-      <c r="H4" t="str" s="24">
-        <v>Jefatura de operaciones</v>
-      </c>
-      <c r="I4" t="str" s="24">
-        <v>2026-08-15</v>
-      </c>
-      <c r="J4" t="str" s="26">
-        <v>implementado</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str" s="23">
-        <v>Recepción, almacenamiento y despacho</v>
-      </c>
-      <c r="B5" t="str" s="23">
-        <v>Operador de bodega</v>
-      </c>
-      <c r="C5" t="str" s="23">
-        <v>Preparar pedidos para despacho</v>
-      </c>
-      <c r="D5" t="str" s="23">
-        <v>B3</v>
-      </c>
-      <c r="E5" t="str" s="23">
-        <v>Cortes por herramientas</v>
-      </c>
-      <c r="F5" t="str" s="23">
-        <v>Administrativo</v>
-      </c>
-      <c r="G5" t="str" s="23">
-        <v>Usar cuchillos de seguridad y capacitar al personal</v>
-      </c>
-      <c r="H5" t="str" s="23">
-        <v>Jefatura de operaciones</v>
-      </c>
-      <c r="I5" t="str" s="23">
-        <v>2026-08-15</v>
-      </c>
-      <c r="J5" t="str" s="25">
-        <v>pendiente</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str" s="24">
-        <v>Recepción, almacenamiento y despacho</v>
-      </c>
-      <c r="B6" t="str" s="24">
-        <v>Operador de bodega</v>
-      </c>
-      <c r="C6" t="str" s="24">
-        <v>Preparar pedidos para despacho</v>
-      </c>
-      <c r="D6" t="str" s="24">
-        <v>B2</v>
-      </c>
-      <c r="E6" t="str" s="24">
-        <v>Caída de objetos</v>
-      </c>
-      <c r="F6" t="str" s="24">
-        <v>Administrativo</v>
-      </c>
-      <c r="G6" t="str" s="24">
-        <v>Reorganizar almacenamiento pesado</v>
-      </c>
-      <c r="H6" t="str" s="24">
-        <v>Jefatura de operaciones</v>
-      </c>
-      <c r="I6" t="str" s="24">
-        <v>2026-08-15</v>
-      </c>
-      <c r="J6" t="str" s="27">
-        <v>en_revision</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str" s="23">
-        <v>Recepción, almacenamiento y despacho</v>
-      </c>
-      <c r="B7" t="str" s="23">
-        <v>Operador de bodega</v>
-      </c>
-      <c r="C7" t="str" s="23">
-        <v>Preparar pedidos para despacho</v>
-      </c>
-      <c r="D7" t="str" s="23">
-        <v>B2</v>
-      </c>
-      <c r="E7" t="str" s="23">
-        <v>Caída de objetos</v>
-      </c>
-      <c r="F7" t="str" s="23">
-        <v>Administrativo</v>
-      </c>
-      <c r="G7" t="str" s="23">
-        <v>Instalar topes de retención</v>
-      </c>
-      <c r="H7" t="str" s="23">
-        <v>Jefatura de operaciones</v>
-      </c>
-      <c r="I7" t="str" s="23">
-        <v>2026-08-15</v>
-      </c>
-      <c r="J7" t="str" s="25">
-        <v>pendiente</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str" s="24">
-        <v>Recepción, almacenamiento y despacho</v>
-      </c>
-      <c r="B8" t="str" s="24">
-        <v>Supervisor de operaciones</v>
-      </c>
-      <c r="C8" t="str" s="24">
-        <v>Gestionar contingencias operacionales</v>
-      </c>
-      <c r="D8" t="str" s="24">
-        <v>F1</v>
-      </c>
-      <c r="E8" t="str" s="24">
-        <v>Contacto eléctrico directo</v>
-      </c>
-      <c r="F8" t="str" s="24">
-        <v>Administrativo</v>
-      </c>
-      <c r="G8" t="str" s="24">
-        <v>Retirar equipo defectuoso y bloquear energías</v>
-      </c>
-      <c r="H8" t="str" s="24">
-        <v>Jefatura de operaciones</v>
-      </c>
-      <c r="I8" t="str" s="24">
-        <v>2026-08-15</v>
-      </c>
-      <c r="J8" t="str" s="25">
-        <v>pendiente</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str" s="23">
-        <v>Recepción, almacenamiento y despacho</v>
-      </c>
-      <c r="B9" t="str" s="23">
-        <v>Operador de bodega</v>
-      </c>
-      <c r="C9" t="str" s="23">
-        <v>Preparar pedidos para despacho</v>
-      </c>
-      <c r="D9" t="str" s="23">
-        <v>P1</v>
-      </c>
-      <c r="E9" t="str" s="23">
-        <v>Exposición a ruido</v>
-      </c>
-      <c r="F9" t="str" s="23">
-        <v>Administrativo</v>
-      </c>
-      <c r="G9" t="str" s="23">
-        <v>Implementar programa de conservación auditiva</v>
-      </c>
-      <c r="H9" t="str" s="23">
-        <v>Jefatura de operaciones</v>
-      </c>
-      <c r="I9" t="str" s="23">
-        <v>2026-08-15</v>
-      </c>
-      <c r="J9" t="str" s="25">
-        <v>pendiente</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str" s="24">
-        <v>Recepción, almacenamiento y despacho</v>
-      </c>
-      <c r="B10" t="str" s="24">
-        <v>Supervisor de operaciones</v>
-      </c>
-      <c r="C10" t="str" s="24">
-        <v>Supervisar operación y coordinar turnos</v>
-      </c>
-      <c r="D10" t="str" s="24">
-        <v>D1</v>
-      </c>
-      <c r="E10" t="str" s="24">
-        <v>Carga de trabajo</v>
-      </c>
-      <c r="F10" t="str" s="24">
-        <v>Administrativo</v>
-      </c>
-      <c r="G10" t="str" s="24">
-        <v>Revisar distribución de carga y pausas</v>
-      </c>
-      <c r="H10" t="str" s="24">
-        <v>Jefatura de operaciones</v>
-      </c>
-      <c r="I10" t="str" s="24">
-        <v>2026-08-15</v>
-      </c>
-      <c r="J10" t="str" s="25">
-        <v>pendiente</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str" s="23">
-        <v>Recepción, almacenamiento y despacho</v>
-      </c>
-      <c r="B11" t="str" s="23">
-        <v>Operador de bodega</v>
-      </c>
-      <c r="C11" t="str" s="23">
-        <v>Recepcionar y almacenar materiales</v>
-      </c>
-      <c r="D11" t="str" s="23">
-        <v>R1</v>
-      </c>
-      <c r="E11" t="str" s="23">
-        <v>Manipulación manual de cargas</v>
-      </c>
-      <c r="F11" t="str" s="23">
-        <v>Administrativo</v>
-      </c>
-      <c r="G11" t="str" s="23">
-        <v>Incorporar ayuda mecánica para cargas</v>
-      </c>
-      <c r="H11" t="str" s="23">
-        <v>Jefatura de operaciones</v>
-      </c>
-      <c r="I11" t="str" s="23">
-        <v>2026-08-15</v>
-      </c>
-      <c r="J11" t="str" s="25">
-        <v>pendiente</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A2:J11"/>
+  <autoFilter ref="A2:J3"/>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J11"/>
-  </ignoredErrors>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.45" header="0.15" footer="0.2"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
@@ -2710,7 +1959,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G3"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -2751,16 +2000,16 @@
     </row>
     <row r="3">
       <c r="A3" t="str" s="23">
-        <v>A1</v>
+        <v>I1</v>
       </c>
       <c r="B3" t="str" s="23">
-        <v>Caída de personas</v>
+        <v>Contacto con / en Vehículos en movimiento</v>
       </c>
       <c r="C3" t="str" s="23">
-        <v>Caídas al mismo nivel</v>
+        <v>Atropellos o golpes con vehículos</v>
       </c>
       <c r="D3" t="str" s="23">
-        <v>Caída que se produce en el mismo plano de sustentación, por ejemplo: caídas en lugares de tránsito o superficies de trabajo, caídas sobre o contra objetos.</v>
+        <v>Impacto entre un peatón y un vehículo en movimiento.</v>
       </c>
       <c r="E3" t="str" s="23">
         <v>seguridad</v>
@@ -2772,153 +2021,11 @@
         <v/>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="str" s="24">
-        <v>B2</v>
-      </c>
-      <c r="B4" t="str" s="24">
-        <v>Contacto con objetos</v>
-      </c>
-      <c r="C4" t="str" s="24">
-        <v>Caída de objetos</v>
-      </c>
-      <c r="D4" t="str" s="24">
-        <v>Caída de elementos que golpean al cuerpo, por ejemplo, materiales, herramientas, estructuras, etc.</v>
-      </c>
-      <c r="E4" t="str" s="24">
-        <v>seguridad</v>
-      </c>
-      <c r="F4" t="str" s="24">
-        <v>vep_isp</v>
-      </c>
-      <c r="G4" t="str" s="24">
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str" s="23">
-        <v>B3</v>
-      </c>
-      <c r="B5" t="str" s="23">
-        <v>Contacto con objetos</v>
-      </c>
-      <c r="C5" t="str" s="23">
-        <v>Cortes por objetos / herramientas corto-punzantes</v>
-      </c>
-      <c r="D5" t="str" s="23">
-        <v>Cortes y/o punzaciones generadas en parte del cuerpo debido al contacto de éste con objetos cortantes, punzantes y/o abrasivos.</v>
-      </c>
-      <c r="E5" t="str" s="23">
-        <v>seguridad</v>
-      </c>
-      <c r="F5" t="str" s="23">
-        <v>vep_isp</v>
-      </c>
-      <c r="G5" t="str" s="23">
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str" s="24">
-        <v>F1</v>
-      </c>
-      <c r="B6" t="str" s="24">
-        <v>Contacto con energía eléctrica</v>
-      </c>
-      <c r="C6" t="str" s="24">
-        <v>Contactos eléctricos directos baja tensión</v>
-      </c>
-      <c r="D6" t="str" s="24">
-        <v>Es todo contacto directo de las personas con partes activas en tensión (trabajando con tensiones menores a 1000 volts).</v>
-      </c>
-      <c r="E6" t="str" s="24">
-        <v>seguridad</v>
-      </c>
-      <c r="F6" t="str" s="24">
-        <v>vep_isp</v>
-      </c>
-      <c r="G6" t="str" s="24">
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str" s="23">
-        <v>P1</v>
-      </c>
-      <c r="B7" t="str" s="23">
-        <v>Exposición a agentes físicos</v>
-      </c>
-      <c r="C7" t="str" s="23">
-        <v>Exposición a ruido</v>
-      </c>
-      <c r="D7" t="str" s="23">
-        <v>Permanencia en un ambiente de trabajo con presencia continua de altos niveles de presión sonora (en forma estable o fluctuante), con la potencialidad de alterar el órgano de la audición.</v>
-      </c>
-      <c r="E7" t="str" s="23">
-        <v>higienico</v>
-      </c>
-      <c r="F7" t="str" s="23">
-        <v>evaluacion_especifica</v>
-      </c>
-      <c r="G7" t="str" s="23">
-        <v>Protocolo de Exposición Ocupacional a Ruido (PREXOR)</v>
-      </c>
-    </row>
-    <row r="8" xml:space="preserve">
-      <c r="A8" t="str" s="24">
-        <v>R1</v>
-      </c>
-      <c r="B8" t="str" s="24">
-        <v>Manejo o Manipulación Manual de Carga (MMC) o personas /Pacientes (MMP)</v>
-      </c>
-      <c r="C8" t="str" s="24">
-        <v>Sobrecarga física debido a la manipulación manual de cargas</v>
-      </c>
-      <c r="D8" t="str" xml:space="preserve" s="24">
-        <v xml:space="preserve">Trabajos en donde se deban levantar, descender o transportar manualmente objetos de más de 3 kilos.
-Trabajos en donde se deban empujar o arrastrar objetos utilizando 1 o 2 manos.</v>
-      </c>
-      <c r="E8" t="str" s="24">
-        <v>musculoesqueletico</v>
-      </c>
-      <c r="F8" t="str" s="24">
-        <v>evaluacion_especifica</v>
-      </c>
-      <c r="G8" t="str" s="24">
-        <v>Guía técnica para la evaluación y control de riesgos asociados al manejo o manipulación manual de carga</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str" s="23">
-        <v>D1</v>
-      </c>
-      <c r="B9" t="str" s="23">
-        <v>Riesgos psicosociales laborales</v>
-      </c>
-      <c r="C9" t="str" s="23">
-        <v>1. Dimensión carga de trabajo (CT).</v>
-      </c>
-      <c r="D9" t="str" s="23">
-        <v>La carga de trabajo son las exigencias que se le hacen a los trabajadores y trabajadoras para que cumplan con un determinado objetivo o tarea en un tiempo acotado o limitado. Es decir, en la carga de trabajo existe una relación entre la cantidad de tareas y el tiempo en que se deben realizar, que puede ser desde minutos hasta semanas o más.</v>
-      </c>
-      <c r="E9" t="str" s="23">
-        <v>psicosocial</v>
-      </c>
-      <c r="F9" t="str" s="23">
-        <v>evaluacion_especifica</v>
-      </c>
-      <c r="G9" t="str" s="23">
-        <v>Protocolo de vigilancia de riesgos psicosociales en el trabajo</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A2:G9"/>
+  <autoFilter ref="A2:G3"/>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G9"/>
-  </ignoredErrors>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.45" header="0.15" footer="0.2"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
@@ -2930,7 +2037,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G7"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -2951,13 +2058,13 @@
         <v>Código</v>
       </c>
       <c r="B2" t="str" s="5">
-        <v>MIPER-PRUEBA-001</v>
+        <v>MIPER-001</v>
       </c>
       <c r="C2" t="str" s="4">
         <v>Versión</v>
       </c>
       <c r="D2" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E2" t="str" s="4">
         <v>Estado</v>
@@ -2971,13 +2078,13 @@
         <v>Versión anterior</v>
       </c>
       <c r="B3" t="str" s="5">
-        <v>No informado</v>
+        <v>MIPER-001-V2</v>
       </c>
       <c r="C3" t="str" s="4">
         <v>Fecha descarga</v>
       </c>
       <c r="D3" t="str" s="5">
-        <v>2026-07-20</v>
+        <v>2026-07-21</v>
       </c>
       <c r="E3" t="str" s="4">
         <v>Nota legacy</v>
@@ -2991,7 +2098,7 @@
         <v>Elaborado por</v>
       </c>
       <c r="B4" t="str" s="5">
-        <v>Diana Marín · Prevencionista de riesgos</v>
+        <v>Ana Perez</v>
       </c>
       <c r="C4" t="str" s="4">
         <v>Revisado por</v>
@@ -3031,16 +2138,16 @@
     </row>
     <row r="7">
       <c r="A7" t="str" s="23">
-        <v>i1</v>
+        <v>i-1</v>
       </c>
       <c r="B7" t="str" s="23">
-        <v>t1</v>
+        <v>t-1</v>
       </c>
       <c r="C7" t="str" s="23">
         <v>vep_isp</v>
       </c>
       <c r="D7" t="str" s="23">
-        <v>Confirmado durante levantamiento ISP</v>
+        <v>Mapeo por exposicion</v>
       </c>
       <c r="E7" t="str" s="23">
         <v>vep</v>
@@ -3049,178 +2156,14 @@
         <v/>
       </c>
       <c r="G7" t="str" s="23">
-        <v>Responsable: Jefatura de operaciones | Protocolo: No informado</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str" s="24">
-        <v>i2</v>
-      </c>
-      <c r="B8" t="str" s="24">
-        <v>t1</v>
-      </c>
-      <c r="C8" t="str" s="24">
-        <v>vep_isp</v>
-      </c>
-      <c r="D8" t="str" s="24">
-        <v>Confirmado durante levantamiento ISP</v>
-      </c>
-      <c r="E8" t="str" s="24">
-        <v>vep</v>
-      </c>
-      <c r="F8" t="str" s="24">
-        <v/>
-      </c>
-      <c r="G8" t="str" s="24">
-        <v>Responsable: Jefatura de operaciones | Protocolo: No informado</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str" s="23">
-        <v>i3</v>
-      </c>
-      <c r="B9" t="str" s="23">
-        <v>t2</v>
-      </c>
-      <c r="C9" t="str" s="23">
-        <v>vep_isp</v>
-      </c>
-      <c r="D9" t="str" s="23">
-        <v>Confirmado durante levantamiento ISP</v>
-      </c>
-      <c r="E9" t="str" s="23">
-        <v>vep</v>
-      </c>
-      <c r="F9" t="str" s="23">
-        <v/>
-      </c>
-      <c r="G9" t="str" s="23">
-        <v>Responsable: Jefatura de operaciones | Protocolo: No informado</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str" s="24">
-        <v>i4</v>
-      </c>
-      <c r="B10" t="str" s="24">
-        <v>t2</v>
-      </c>
-      <c r="C10" t="str" s="24">
-        <v>vep_isp</v>
-      </c>
-      <c r="D10" t="str" s="24">
-        <v>Confirmado durante levantamiento ISP</v>
-      </c>
-      <c r="E10" t="str" s="24">
-        <v>vep</v>
-      </c>
-      <c r="F10" t="str" s="24">
-        <v/>
-      </c>
-      <c r="G10" t="str" s="24">
-        <v>Responsable: Jefatura de operaciones | Protocolo: No informado</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str" s="23">
-        <v>i5</v>
-      </c>
-      <c r="B11" t="str" s="23">
-        <v>t4</v>
-      </c>
-      <c r="C11" t="str" s="23">
-        <v>vep_isp</v>
-      </c>
-      <c r="D11" t="str" s="23">
-        <v>Confirmado durante levantamiento ISP</v>
-      </c>
-      <c r="E11" t="str" s="23">
-        <v>vep</v>
-      </c>
-      <c r="F11" t="str" s="23">
-        <v/>
-      </c>
-      <c r="G11" t="str" s="23">
-        <v>Responsable: Jefatura de operaciones | Protocolo: No informado</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str" s="24">
-        <v>i6</v>
-      </c>
-      <c r="B12" t="str" s="24">
-        <v>t2</v>
-      </c>
-      <c r="C12" t="str" s="24">
-        <v>evaluacion_especifica</v>
-      </c>
-      <c r="D12" t="str" s="24">
-        <v>Confirmado durante levantamiento ISP</v>
-      </c>
-      <c r="E12" t="str" s="24">
-        <v>evaluado</v>
-      </c>
-      <c r="F12" t="str" s="24">
-        <v>Medición higiénica programada</v>
-      </c>
-      <c r="G12" t="str" s="24">
-        <v>Responsable: Jefatura de operaciones | Protocolo: PREXOR</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str" s="23">
-        <v>i7</v>
-      </c>
-      <c r="B13" t="str" s="23">
-        <v>t3</v>
-      </c>
-      <c r="C13" t="str" s="23">
-        <v>evaluacion_especifica</v>
-      </c>
-      <c r="D13" t="str" s="23">
-        <v>Confirmado durante levantamiento ISP</v>
-      </c>
-      <c r="E13" t="str" s="23">
-        <v>evaluado</v>
-      </c>
-      <c r="F13" t="str" s="23">
-        <v>Resultado por unidad</v>
-      </c>
-      <c r="G13" t="str" s="23">
-        <v>Responsable: Jefatura de operaciones | Protocolo: CEAL-SM/SUSESO</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str" s="24">
-        <v>i8</v>
-      </c>
-      <c r="B14" t="str" s="24">
-        <v>t1</v>
-      </c>
-      <c r="C14" t="str" s="24">
-        <v>evaluacion_especifica</v>
-      </c>
-      <c r="D14" t="str" s="24">
-        <v>Confirmado durante levantamiento ISP</v>
-      </c>
-      <c r="E14" t="str" s="24">
-        <v>evaluado</v>
-      </c>
-      <c r="F14" t="str" s="24">
-        <v>Evaluación inicial</v>
-      </c>
-      <c r="G14" t="str" s="24">
-        <v>Responsable: Jefatura de operaciones | Protocolo: MMC</v>
+        <v>Responsable: Juan Soto | Protocolo: No informado</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:G14"/>
+  <autoFilter ref="A6:G7"/>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G14"/>
-  </ignoredErrors>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.45" header="0.15" footer="0.2"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
fix: corrige Excel y responsables MIPER (#83)
Co-authored-by: DICAPREV <dicaprev@iMac-de-DICAPREV.local>
</commit_message>
<xml_diff>
--- a/docs/evidencias-ds44-miper/MIPER-NEXTPREV-MIPER-PRUEBA-001-V1.xlsx
+++ b/docs/evidencias-ds44-miper/MIPER-NEXTPREV-MIPER-PRUEBA-001-V1.xlsx
@@ -11,7 +11,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">MIPER!$11:$13</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">MIPER!$A$1:$P$27</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">MIPER!$A$1:$P$20</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -664,7 +664,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P27"/>
+  <dimension ref="A1:P20"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -839,7 +839,7 @@
         <v>Código</v>
       </c>
       <c r="B4" t="str" s="5">
-        <v>MIPER-PRUEBA-001</v>
+        <v>MIPER-001</v>
       </c>
       <c r="C4" t="str" s="5">
         <v/>
@@ -851,7 +851,7 @@
         <v>Versión</v>
       </c>
       <c r="F4" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G4" t="str" s="5">
         <v/>
@@ -889,7 +889,7 @@
         <v>Entidad empleadora</v>
       </c>
       <c r="B5" t="str" s="5">
-        <v>Empresa demostrativa NextPrev</v>
+        <v>Empresa Demo</v>
       </c>
       <c r="C5" t="str" s="5">
         <v/>
@@ -913,7 +913,7 @@
         <v>Centro de trabajo</v>
       </c>
       <c r="J5" t="str" s="5">
-        <v>Casa matriz / Principal</v>
+        <v>Centro Norte</v>
       </c>
       <c r="K5" t="str" s="5">
         <v/>
@@ -939,7 +939,7 @@
         <v>Proceso</v>
       </c>
       <c r="B6" t="str" s="5">
-        <v>Recepción, almacenamiento y despacho</v>
+        <v>Operacion mina</v>
       </c>
       <c r="C6" t="str" s="5">
         <v/>
@@ -963,7 +963,7 @@
         <v>Responsable proceso</v>
       </c>
       <c r="J6" t="str" s="5">
-        <v>Jefatura de operaciones</v>
+        <v>Camila Soto</v>
       </c>
       <c r="K6" t="str" s="5">
         <v/>
@@ -1086,43 +1086,43 @@
     </row>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B9" t="str" s="7">
         <v/>
       </c>
       <c r="C9" s="7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D9" t="str" s="7">
         <v/>
       </c>
       <c r="E9" s="7">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F9" t="str" s="7">
         <v/>
       </c>
       <c r="G9" s="7">
+        <v>0</v>
+      </c>
+      <c r="H9" t="str" s="7">
+        <v/>
+      </c>
+      <c r="I9" s="7">
         <v>1</v>
       </c>
-      <c r="H9" t="str" s="7">
-        <v/>
-      </c>
-      <c r="I9" s="7">
-        <v>7</v>
-      </c>
       <c r="J9" t="str" s="7">
         <v/>
       </c>
       <c r="K9" s="7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L9" t="str" s="7">
         <v/>
       </c>
       <c r="M9" s="7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N9" t="str" s="7">
         <v/>
@@ -1336,31 +1336,33 @@
     </row>
     <row r="14" xml:space="preserve">
       <c r="A14" t="str" s="11">
-        <v>Recepción, almacenamiento y despacho</v>
+        <v>Operacion mina</v>
       </c>
       <c r="B14" t="str" s="11">
-        <v>Operador de bodega</v>
+        <v>Operador</v>
       </c>
       <c r="C14" t="str" s="11">
-        <v>Recepcionar y almacenar materiales</v>
+        <v>Traslado interno</v>
       </c>
       <c r="D14" t="str" s="11">
-        <v>Gente: Personas expuestas durante la tarea | Equipos: Equipos móviles y herramientas | Materiales: Materiales almacenados | Ambiente: Superficie y condiciones del lugar | Detalle: Interacción observable durante la ejecución</v>
+        <v>Gente: Conductor fatigado | Equipos: Camioneta en maniobra | Detalle: Cruce sin demarcacion</v>
       </c>
       <c r="E14" t="str" s="11">
-        <v>Caídas al mismo nivel (A1)</v>
-      </c>
-      <c r="F14" t="str" s="11">
-        <v/>
-      </c>
-      <c r="G14" t="str" s="11">
-        <v/>
-      </c>
-      <c r="H14" t="str" s="11">
-        <v/>
-      </c>
-      <c r="I14" t="str" s="13">
-        <v/>
+        <v>Atropello (I1)</v>
+      </c>
+      <c r="F14" s="11">
+        <v>2</v>
+      </c>
+      <c r="G14" s="11">
+        <v>2</v>
+      </c>
+      <c r="H14" s="11">
+        <f>F14*G14</f>
+        <v>4</v>
+      </c>
+      <c r="I14" t="str" s="11">
+        <f>IF(H14&lt;=2,"Tolerable",IF(H14=4,"Moderado",IF(H14=8,"Importante","Intolerable")))</f>
+        <v>Moderado</v>
       </c>
       <c r="J14" t="str" s="11">
         <v/>
@@ -1381,597 +1383,214 @@
         <v/>
       </c>
       <c r="P14" t="str" xml:space="preserve" s="11">
-        <v xml:space="preserve">Administrativo: Demarcar rutas y verificar orden y limpieza
-Responsable: Jefatura de operaciones
-Plazo: 2026-08-15
+        <v xml:space="preserve">Administrativo: Control de velocidad
+Responsable: Juan Soto
+Plazo: 2026-07-20
 Estado: pendiente</v>
       </c>
     </row>
-    <row r="15" xml:space="preserve">
-      <c r="A15" t="str" s="12">
-        <v>Recepción, almacenamiento y despacho</v>
-      </c>
-      <c r="B15" t="str" s="12">
-        <v>Operador de bodega</v>
-      </c>
-      <c r="C15" t="str" s="12">
-        <v>Recepcionar y almacenar materiales</v>
-      </c>
-      <c r="D15" t="str" s="12">
-        <v>Gente: Personas expuestas durante la tarea | Equipos: Equipos móviles y herramientas | Materiales: Materiales almacenados | Ambiente: Superficie y condiciones del lugar | Detalle: Interacción observable durante la ejecución</v>
-      </c>
-      <c r="E15" t="str" s="12">
-        <v>Caídas al mismo nivel (A1)</v>
-      </c>
-      <c r="F15" s="12">
-        <v>1</v>
-      </c>
-      <c r="G15" s="12">
-        <v>2</v>
-      </c>
-      <c r="H15" s="12">
-        <f>F15*G15</f>
-        <v>2</v>
-      </c>
-      <c r="I15" t="str" s="12">
-        <f>IF(H15&lt;=2,"Tolerable",IF(H15=4,"Moderado",IF(H15=8,"Importante","Intolerable")))</f>
-        <v>Tolerable</v>
-      </c>
-      <c r="J15" t="str" s="12">
-        <v/>
-      </c>
-      <c r="K15" t="str" s="12">
-        <v/>
-      </c>
-      <c r="L15" t="str" s="12">
-        <v/>
-      </c>
-      <c r="M15" t="str" s="12">
-        <v/>
-      </c>
-      <c r="N15" t="str" s="12">
-        <v/>
-      </c>
-      <c r="O15" t="str" s="12">
-        <v/>
-      </c>
-      <c r="P15" t="str" xml:space="preserve" s="12">
-        <v xml:space="preserve">Administrativo: Inspección diaria de superficies
-Responsable: Jefatura de operaciones
-Plazo: 2026-08-15
-Estado: implementado</v>
-      </c>
-    </row>
-    <row r="16" xml:space="preserve">
-      <c r="A16" t="str" s="29">
-        <v>Recepción, almacenamiento y despacho</v>
-      </c>
-      <c r="B16" t="str" s="29">
-        <v>Operador de bodega</v>
-      </c>
-      <c r="C16" t="str" s="29">
-        <v>Preparar pedidos para despacho</v>
-      </c>
-      <c r="D16" t="str" s="29">
-        <v>Gente: Personas expuestas durante la tarea | Equipos: Equipos móviles y herramientas | Materiales: Materiales almacenados | Ambiente: Superficie y condiciones del lugar | Detalle: Interacción observable durante la ejecución</v>
-      </c>
-      <c r="E16" t="str" s="29">
-        <v>Cortes por herramientas (B3)</v>
-      </c>
-      <c r="F16" s="29">
-        <v>2</v>
-      </c>
-      <c r="G16" s="29">
-        <v>2</v>
-      </c>
-      <c r="H16" s="29">
-        <f>F16*G16</f>
-        <v>4</v>
-      </c>
-      <c r="I16" t="str" s="29">
-        <f>IF(H16&lt;=2,"Tolerable",IF(H16=4,"Moderado",IF(H16=8,"Importante","Intolerable")))</f>
-        <v>Moderado</v>
-      </c>
-      <c r="J16" t="str" s="29">
-        <v/>
-      </c>
-      <c r="K16" t="str" s="29">
-        <v/>
-      </c>
-      <c r="L16" t="str" s="29">
-        <v/>
-      </c>
-      <c r="M16" t="str" s="29">
-        <v/>
-      </c>
-      <c r="N16" t="str" s="29">
-        <v/>
-      </c>
-      <c r="O16" t="str" s="29">
-        <v/>
-      </c>
-      <c r="P16" t="str" xml:space="preserve" s="29">
-        <v xml:space="preserve">Administrativo: Usar cuchillos de seguridad y capacitar al personal
-Responsable: Jefatura de operaciones
-Plazo: 2026-08-15
-Estado: pendiente</v>
-      </c>
-    </row>
-    <row r="17" xml:space="preserve">
-      <c r="A17" t="str" s="12">
-        <v>Recepción, almacenamiento y despacho</v>
-      </c>
-      <c r="B17" t="str" s="12">
-        <v>Operador de bodega</v>
-      </c>
-      <c r="C17" t="str" s="12">
-        <v>Preparar pedidos para despacho</v>
-      </c>
-      <c r="D17" t="str" s="12">
-        <v>Gente: Personas expuestas durante la tarea | Equipos: Equipos móviles y herramientas | Materiales: Materiales almacenados | Ambiente: Superficie y condiciones del lugar | Detalle: Interacción observable durante la ejecución</v>
-      </c>
-      <c r="E17" t="str" s="12">
-        <v>Caída de objetos (B2)</v>
-      </c>
-      <c r="F17" s="12">
-        <v>2</v>
-      </c>
-      <c r="G17" s="12">
-        <v>4</v>
-      </c>
-      <c r="H17" s="12">
-        <f>F17*G17</f>
-        <v>8</v>
-      </c>
-      <c r="I17" t="str" s="12">
-        <f>IF(H17&lt;=2,"Tolerable",IF(H17=4,"Moderado",IF(H17=8,"Importante","Intolerable")))</f>
-        <v>Importante</v>
-      </c>
-      <c r="J17" t="str" s="12">
-        <v/>
-      </c>
-      <c r="K17" t="str" s="12">
-        <v/>
-      </c>
-      <c r="L17" t="str" s="12">
-        <v/>
-      </c>
-      <c r="M17" t="str" s="12">
-        <v/>
-      </c>
-      <c r="N17" t="str" s="12">
-        <v/>
-      </c>
-      <c r="O17" t="str" s="12">
-        <v/>
-      </c>
-      <c r="P17" t="str" xml:space="preserve" s="12">
-        <v xml:space="preserve">Administrativo: Reorganizar almacenamiento pesado
-Responsable: Jefatura de operaciones
-Plazo: 2026-08-15
-Estado: en_revision
-Administrativo: Instalar topes de retención
-Responsable: Jefatura de operaciones
-Plazo: 2026-08-15
-Estado: pendiente</v>
-      </c>
-    </row>
-    <row r="18" xml:space="preserve">
-      <c r="A18" t="str" s="29">
-        <v>Recepción, almacenamiento y despacho</v>
-      </c>
-      <c r="B18" t="str" s="29">
-        <v>Supervisor de operaciones</v>
-      </c>
-      <c r="C18" t="str" s="29">
-        <v>Gestionar contingencias operacionales</v>
-      </c>
-      <c r="D18" t="str" s="29">
-        <v>Gente: Personas expuestas durante la tarea | Equipos: Equipos móviles y herramientas | Materiales: Materiales almacenados | Ambiente: Superficie y condiciones del lugar | Detalle: Interacción observable durante la ejecución</v>
-      </c>
-      <c r="E18" t="str" s="29">
-        <v>Contacto eléctrico directo (F1)</v>
-      </c>
-      <c r="F18" s="29">
-        <v>4</v>
-      </c>
-      <c r="G18" s="29">
-        <v>4</v>
-      </c>
-      <c r="H18" s="29">
-        <f>F18*G18</f>
-        <v>16</v>
-      </c>
-      <c r="I18" t="str" s="29">
-        <f>IF(H18&lt;=2,"Tolerable",IF(H18=4,"Moderado",IF(H18=8,"Importante","Intolerable")))</f>
-        <v>Intolerable</v>
-      </c>
-      <c r="J18" t="str" s="29">
-        <v/>
-      </c>
-      <c r="K18" t="str" s="29">
-        <v/>
-      </c>
-      <c r="L18" t="str" s="29">
-        <v/>
-      </c>
-      <c r="M18" t="str" s="29">
-        <v/>
-      </c>
-      <c r="N18" t="str" s="29">
-        <v/>
-      </c>
-      <c r="O18" t="str" s="29">
-        <v/>
-      </c>
-      <c r="P18" t="str" xml:space="preserve" s="29">
-        <v xml:space="preserve">Administrativo: Retirar equipo defectuoso y bloquear energías
-Responsable: Jefatura de operaciones
-Plazo: 2026-08-15
-Estado: pendiente</v>
-      </c>
-    </row>
-    <row r="19" xml:space="preserve">
-      <c r="A19" t="str" s="30">
-        <v>Recepción, almacenamiento y despacho</v>
-      </c>
-      <c r="B19" t="str" s="30">
-        <v>Operador de bodega</v>
-      </c>
-      <c r="C19" t="str" s="30">
-        <v>Preparar pedidos para despacho</v>
-      </c>
-      <c r="D19" t="str" s="30">
-        <v>Gente: Personas expuestas durante la tarea | Equipos: Equipos móviles y herramientas | Materiales: Materiales almacenados | Ambiente: Superficie y condiciones del lugar | Detalle: Interacción observable durante la ejecución</v>
-      </c>
-      <c r="E19" t="str" s="30">
-        <v>Exposición a ruido (P1)</v>
-      </c>
-      <c r="F19" t="str" s="30">
-        <v/>
-      </c>
-      <c r="G19" t="str" s="30">
-        <v/>
-      </c>
-      <c r="H19" t="str" s="30">
-        <v/>
-      </c>
-      <c r="I19" t="str" s="30">
-        <v/>
-      </c>
-      <c r="J19" t="str" s="30">
-        <v>83 dB(A)</v>
-      </c>
-      <c r="K19" t="str" s="30">
-        <v>Sobre criterio de acción</v>
-      </c>
-      <c r="L19" t="str" s="30">
-        <v/>
-      </c>
-      <c r="M19" t="str" s="30">
-        <v/>
-      </c>
-      <c r="N19" t="str" s="30">
-        <v/>
-      </c>
-      <c r="O19" t="str" s="30">
-        <v/>
-      </c>
-      <c r="P19" t="str" xml:space="preserve" s="30">
-        <v xml:space="preserve">Administrativo: Implementar programa de conservación auditiva
-Responsable: Jefatura de operaciones
-Plazo: 2026-08-15
-Estado: pendiente</v>
-      </c>
-    </row>
-    <row r="20" xml:space="preserve">
-      <c r="A20" t="str" s="29">
-        <v>Recepción, almacenamiento y despacho</v>
-      </c>
-      <c r="B20" t="str" s="29">
-        <v>Supervisor de operaciones</v>
-      </c>
-      <c r="C20" t="str" s="29">
-        <v>Supervisar operación y coordinar turnos</v>
-      </c>
-      <c r="D20" t="str" s="29">
-        <v>Gente: Personas expuestas durante la tarea | Equipos: Equipos móviles y herramientas | Materiales: Materiales almacenados | Ambiente: Superficie y condiciones del lugar | Detalle: Interacción observable durante la ejecución</v>
-      </c>
-      <c r="E20" t="str" s="29">
-        <v>Carga de trabajo (D1)</v>
-      </c>
-      <c r="F20" t="str" s="29">
-        <v/>
-      </c>
-      <c r="G20" t="str" s="29">
-        <v/>
-      </c>
-      <c r="H20" t="str" s="29">
-        <v/>
-      </c>
-      <c r="I20" t="str" s="29">
-        <v/>
-      </c>
-      <c r="J20" t="str" s="29">
-        <v/>
-      </c>
-      <c r="K20" t="str" s="29">
-        <v/>
-      </c>
-      <c r="L20" t="str" s="29">
-        <v>CEAL-SM/SUSESO</v>
-      </c>
-      <c r="M20" t="str" s="29">
-        <v>Riesgo medio</v>
-      </c>
-      <c r="N20" t="str" s="29">
-        <v/>
-      </c>
-      <c r="O20" t="str" s="29">
-        <v/>
-      </c>
-      <c r="P20" t="str" xml:space="preserve" s="29">
-        <v xml:space="preserve">Administrativo: Revisar distribución de carga y pausas
-Responsable: Jefatura de operaciones
-Plazo: 2026-08-15
-Estado: pendiente</v>
-      </c>
-    </row>
-    <row r="21" xml:space="preserve">
-      <c r="A21" t="str" s="30">
-        <v>Recepción, almacenamiento y despacho</v>
-      </c>
-      <c r="B21" t="str" s="30">
-        <v>Operador de bodega</v>
-      </c>
-      <c r="C21" t="str" s="30">
-        <v>Recepcionar y almacenar materiales</v>
-      </c>
-      <c r="D21" t="str" s="30">
-        <v>Gente: Personas expuestas durante la tarea | Equipos: Equipos móviles y herramientas | Materiales: Materiales almacenados | Ambiente: Superficie y condiciones del lugar | Detalle: Interacción observable durante la ejecución</v>
-      </c>
-      <c r="E21" t="str" s="30">
-        <v>Manipulación manual de cargas (R1)</v>
-      </c>
-      <c r="F21" t="str" s="30">
-        <v/>
-      </c>
-      <c r="G21" t="str" s="30">
-        <v/>
-      </c>
-      <c r="H21" t="str" s="30">
-        <v/>
-      </c>
-      <c r="I21" t="str" s="30">
-        <v/>
-      </c>
-      <c r="J21" t="str" s="30">
-        <v/>
-      </c>
-      <c r="K21" t="str" s="30">
-        <v/>
-      </c>
-      <c r="L21" t="str" s="30">
-        <v/>
-      </c>
-      <c r="M21" t="str" s="30">
-        <v/>
-      </c>
-      <c r="N21" t="str" s="30">
-        <v>MAC nivel 3</v>
-      </c>
-      <c r="O21" t="str" s="30">
-        <v>Alto</v>
-      </c>
-      <c r="P21" t="str" xml:space="preserve" s="30">
-        <v xml:space="preserve">Administrativo: Incorporar ayuda mecánica para cargas
-Responsable: Jefatura de operaciones
-Plazo: 2026-08-15
-Estado: pendiente</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str" s="19">
+    <row r="16">
+      <c r="A16" t="str" s="19">
         <v>Firmas y aprobación</v>
       </c>
-      <c r="B23" t="str" s="19">
-        <v/>
-      </c>
-      <c r="C23" t="str" s="19">
-        <v/>
-      </c>
-      <c r="D23" t="str" s="19">
-        <v/>
-      </c>
-      <c r="E23" t="str" s="19">
-        <v/>
-      </c>
-      <c r="F23" t="str" s="19">
-        <v/>
-      </c>
-      <c r="G23" t="str" s="19">
-        <v/>
-      </c>
-      <c r="H23" t="str" s="19">
-        <v/>
-      </c>
-      <c r="I23" t="str" s="19">
-        <v/>
-      </c>
-      <c r="J23" t="str" s="19">
-        <v/>
-      </c>
-      <c r="K23" t="str" s="19">
-        <v/>
-      </c>
-      <c r="L23" t="str" s="19">
-        <v/>
-      </c>
-      <c r="M23" t="str" s="19">
-        <v/>
-      </c>
-      <c r="N23" t="str" s="19">
-        <v/>
-      </c>
-      <c r="O23" t="str" s="19">
-        <v/>
-      </c>
-      <c r="P23" t="str" s="19">
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="str" s="20">
+      <c r="B16" t="str" s="19">
+        <v/>
+      </c>
+      <c r="C16" t="str" s="19">
+        <v/>
+      </c>
+      <c r="D16" t="str" s="19">
+        <v/>
+      </c>
+      <c r="E16" t="str" s="19">
+        <v/>
+      </c>
+      <c r="F16" t="str" s="19">
+        <v/>
+      </c>
+      <c r="G16" t="str" s="19">
+        <v/>
+      </c>
+      <c r="H16" t="str" s="19">
+        <v/>
+      </c>
+      <c r="I16" t="str" s="19">
+        <v/>
+      </c>
+      <c r="J16" t="str" s="19">
+        <v/>
+      </c>
+      <c r="K16" t="str" s="19">
+        <v/>
+      </c>
+      <c r="L16" t="str" s="19">
+        <v/>
+      </c>
+      <c r="M16" t="str" s="19">
+        <v/>
+      </c>
+      <c r="N16" t="str" s="19">
+        <v/>
+      </c>
+      <c r="O16" t="str" s="19">
+        <v/>
+      </c>
+      <c r="P16" t="str" s="19">
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str" s="20">
         <v>Elaborado por</v>
       </c>
-      <c r="B25" t="str" s="5">
-        <v>Diana Marín · Prevencionista de riesgos</v>
-      </c>
-      <c r="C25" t="str" s="5">
-        <v/>
-      </c>
-      <c r="D25" t="str" s="5">
-        <v/>
-      </c>
-      <c r="E25" t="str" s="5">
-        <v/>
-      </c>
-      <c r="F25" t="str" s="20">
+      <c r="B18" t="str" s="5">
+        <v>Ana Perez</v>
+      </c>
+      <c r="C18" t="str" s="5">
+        <v/>
+      </c>
+      <c r="D18" t="str" s="5">
+        <v/>
+      </c>
+      <c r="E18" t="str" s="5">
+        <v/>
+      </c>
+      <c r="F18" t="str" s="20">
         <v>Fecha</v>
       </c>
-      <c r="G25" t="str" s="5">
+      <c r="G18" t="str" s="5">
         <v>2026-07-20</v>
       </c>
-      <c r="H25" t="str" s="5">
-        <v/>
-      </c>
-      <c r="I25" t="str" s="20">
+      <c r="H18" t="str" s="5">
+        <v/>
+      </c>
+      <c r="I18" t="str" s="20">
         <v>Revisado por</v>
       </c>
-      <c r="J25" t="str" s="5">
+      <c r="J18" t="str" s="5">
         <v>No informado</v>
       </c>
-      <c r="K25" t="str" s="5">
-        <v/>
-      </c>
-      <c r="L25" t="str" s="5">
-        <v/>
-      </c>
-      <c r="M25" t="str" s="20">
+      <c r="K18" t="str" s="5">
+        <v/>
+      </c>
+      <c r="L18" t="str" s="5">
+        <v/>
+      </c>
+      <c r="M18" t="str" s="20">
         <v>Fecha</v>
       </c>
-      <c r="N25" t="str" s="5">
+      <c r="N18" t="str" s="5">
         <v>Pendiente</v>
       </c>
-      <c r="O25" t="str" s="5">
-        <v/>
-      </c>
-      <c r="P25" t="str" s="5">
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="str" s="20">
+      <c r="O18" t="str" s="5">
+        <v/>
+      </c>
+      <c r="P18" t="str" s="5">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str" s="20">
         <v>Cargo / rol</v>
       </c>
-      <c r="B26" t="str" s="5">
+      <c r="B19" t="str" s="5">
         <v>Prevención de riesgos</v>
       </c>
-      <c r="C26" t="str" s="5">
-        <v/>
-      </c>
-      <c r="D26" t="str" s="5">
-        <v/>
-      </c>
-      <c r="E26" t="str" s="5">
-        <v/>
-      </c>
-      <c r="F26" t="str" s="20">
-        <v/>
-      </c>
-      <c r="G26" t="str" s="5">
-        <v/>
-      </c>
-      <c r="H26" t="str" s="5">
-        <v/>
-      </c>
-      <c r="I26" t="str" s="20">
+      <c r="C19" t="str" s="5">
+        <v/>
+      </c>
+      <c r="D19" t="str" s="5">
+        <v/>
+      </c>
+      <c r="E19" t="str" s="5">
+        <v/>
+      </c>
+      <c r="F19" t="str" s="20">
+        <v/>
+      </c>
+      <c r="G19" t="str" s="5">
+        <v/>
+      </c>
+      <c r="H19" t="str" s="5">
+        <v/>
+      </c>
+      <c r="I19" t="str" s="20">
         <v>Cargo / rol</v>
       </c>
-      <c r="J26" t="str" s="5">
+      <c r="J19" t="str" s="5">
         <v>Pendiente</v>
       </c>
-      <c r="K26" t="str" s="5">
-        <v/>
-      </c>
-      <c r="L26" t="str" s="5">
-        <v/>
-      </c>
-      <c r="M26" t="str" s="20">
-        <v/>
-      </c>
-      <c r="N26" t="str" s="5">
-        <v/>
-      </c>
-      <c r="O26" t="str" s="5">
-        <v/>
-      </c>
-      <c r="P26" t="str" s="5">
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="str" s="20">
+      <c r="K19" t="str" s="5">
+        <v/>
+      </c>
+      <c r="L19" t="str" s="5">
+        <v/>
+      </c>
+      <c r="M19" t="str" s="20">
+        <v/>
+      </c>
+      <c r="N19" t="str" s="5">
+        <v/>
+      </c>
+      <c r="O19" t="str" s="5">
+        <v/>
+      </c>
+      <c r="P19" t="str" s="5">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str" s="20">
         <v>Aprobado por</v>
       </c>
-      <c r="B27" t="str" s="5">
+      <c r="B20" t="str" s="5">
         <v>No informado</v>
       </c>
-      <c r="C27" t="str" s="5">
-        <v/>
-      </c>
-      <c r="D27" t="str" s="5">
-        <v/>
-      </c>
-      <c r="E27" t="str" s="5">
-        <v/>
-      </c>
-      <c r="F27" t="str" s="20">
+      <c r="C20" t="str" s="5">
+        <v/>
+      </c>
+      <c r="D20" t="str" s="5">
+        <v/>
+      </c>
+      <c r="E20" t="str" s="5">
+        <v/>
+      </c>
+      <c r="F20" t="str" s="20">
         <v>Fecha</v>
       </c>
-      <c r="G27" t="str" s="5">
+      <c r="G20" t="str" s="5">
         <v>Pendiente</v>
       </c>
-      <c r="H27" t="str" s="5">
-        <v/>
-      </c>
-      <c r="I27" t="str" s="20">
+      <c r="H20" t="str" s="5">
+        <v/>
+      </c>
+      <c r="I20" t="str" s="20">
         <v>Cargo / rol</v>
       </c>
-      <c r="J27" t="str" s="5">
+      <c r="J20" t="str" s="5">
         <v>Pendiente</v>
       </c>
-      <c r="K27" t="str" s="5">
-        <v/>
-      </c>
-      <c r="L27" t="str" s="5">
-        <v/>
-      </c>
-      <c r="M27" t="str" s="20">
-        <v/>
-      </c>
-      <c r="N27" t="str" s="5">
-        <v/>
-      </c>
-      <c r="O27" t="str" s="5">
-        <v/>
-      </c>
-      <c r="P27" t="str" s="5">
+      <c r="K20" t="str" s="5">
+        <v/>
+      </c>
+      <c r="L20" t="str" s="5">
+        <v/>
+      </c>
+      <c r="M20" t="str" s="20">
+        <v/>
+      </c>
+      <c r="N20" t="str" s="5">
+        <v/>
+      </c>
+      <c r="O20" t="str" s="5">
+        <v/>
+      </c>
+      <c r="P20" t="str" s="5">
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A13:P21"/>
+  <autoFilter ref="A13:P14"/>
   <mergeCells count="50">
     <mergeCell ref="A1:C2"/>
     <mergeCell ref="D1:P2"/>
@@ -2010,119 +1629,116 @@
     <mergeCell ref="J12:K12"/>
     <mergeCell ref="L12:M12"/>
     <mergeCell ref="N12:O12"/>
-    <mergeCell ref="A23:P23"/>
-    <mergeCell ref="B25:E25"/>
-    <mergeCell ref="G25:H25"/>
-    <mergeCell ref="J25:L25"/>
-    <mergeCell ref="N25:P25"/>
-    <mergeCell ref="B26:E26"/>
-    <mergeCell ref="G26:H26"/>
-    <mergeCell ref="J26:L26"/>
-    <mergeCell ref="N26:P26"/>
-    <mergeCell ref="B27:E27"/>
-    <mergeCell ref="G27:H27"/>
-    <mergeCell ref="J27:L27"/>
-    <mergeCell ref="N27:P27"/>
+    <mergeCell ref="A16:P16"/>
+    <mergeCell ref="B18:E18"/>
+    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="J18:L18"/>
+    <mergeCell ref="N18:P18"/>
+    <mergeCell ref="B19:E19"/>
+    <mergeCell ref="G19:H19"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="N19:P19"/>
+    <mergeCell ref="B20:E20"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="J20:L20"/>
+    <mergeCell ref="N20:P20"/>
   </mergeCells>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P27"/>
-  </ignoredErrors>
-  <conditionalFormatting sqref="I14:I21">
+  <conditionalFormatting sqref="I14:I14">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>EXACT(I14,"Evaluación pendiente")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I14:I21">
+  <conditionalFormatting sqref="I14:I14">
     <cfRule type="expression" dxfId="1" priority="2">
       <formula>EXACT(I14,"Tolerable")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I14:I21">
+  <conditionalFormatting sqref="I14:I14">
     <cfRule type="expression" dxfId="2" priority="3">
       <formula>EXACT(I14,"Moderado")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I14:I21">
+  <conditionalFormatting sqref="I14:I14">
     <cfRule type="expression" dxfId="3" priority="4">
       <formula>EXACT(I14,"Importante")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I14:I21">
+  <conditionalFormatting sqref="I14:I14">
     <cfRule type="expression" dxfId="4" priority="5">
       <formula>EXACT(I14,"Intolerable")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K14:K21">
+  <conditionalFormatting sqref="K14:K14">
     <cfRule type="expression" dxfId="0" priority="6">
       <formula>EXACT(K14,"Evaluación pendiente")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K14:K21">
+  <conditionalFormatting sqref="K14:K14">
     <cfRule type="expression" dxfId="1" priority="7">
       <formula>EXACT(K14,"Tolerable")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K14:K21">
+  <conditionalFormatting sqref="K14:K14">
     <cfRule type="expression" dxfId="2" priority="8">
       <formula>EXACT(K14,"Moderado")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K14:K21">
+  <conditionalFormatting sqref="K14:K14">
     <cfRule type="expression" dxfId="3" priority="9">
       <formula>EXACT(K14,"Importante")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K14:K21">
+  <conditionalFormatting sqref="K14:K14">
     <cfRule type="expression" dxfId="4" priority="10">
       <formula>EXACT(K14,"Intolerable")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M14:M21">
+  <conditionalFormatting sqref="M14:M14">
     <cfRule type="expression" dxfId="0" priority="11">
       <formula>EXACT(M14,"Evaluación pendiente")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M14:M21">
+  <conditionalFormatting sqref="M14:M14">
     <cfRule type="expression" dxfId="1" priority="12">
       <formula>EXACT(M14,"Tolerable")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M14:M21">
+  <conditionalFormatting sqref="M14:M14">
     <cfRule type="expression" dxfId="2" priority="13">
       <formula>EXACT(M14,"Moderado")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M14:M21">
+  <conditionalFormatting sqref="M14:M14">
     <cfRule type="expression" dxfId="3" priority="14">
       <formula>EXACT(M14,"Importante")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M14:M21">
+  <conditionalFormatting sqref="M14:M14">
     <cfRule type="expression" dxfId="4" priority="15">
       <formula>EXACT(M14,"Intolerable")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O14:O21">
+  <conditionalFormatting sqref="O14:O14">
     <cfRule type="expression" dxfId="0" priority="16">
       <formula>EXACT(O14,"Evaluación pendiente")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O14:O21">
+  <conditionalFormatting sqref="O14:O14">
     <cfRule type="expression" dxfId="1" priority="17">
       <formula>EXACT(O14,"Tolerable")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O14:O21">
+  <conditionalFormatting sqref="O14:O14">
     <cfRule type="expression" dxfId="2" priority="18">
       <formula>EXACT(O14,"Moderado")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O14:O21">
+  <conditionalFormatting sqref="O14:O14">
     <cfRule type="expression" dxfId="3" priority="19">
       <formula>EXACT(O14,"Importante")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O14:O21">
+  <conditionalFormatting sqref="O14:O14">
     <cfRule type="expression" dxfId="4" priority="20">
       <formula>EXACT(O14,"Intolerable")</formula>
     </cfRule>
@@ -2131,14 +1747,14 @@
   <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.45" header="0.15" footer="0.2"/>
   <pageSetup paperSize="8" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
   <headerFooter>
-    <oddFooter>MIPER-PRUEBA-001 V1 | borrador | 2026-07-20 | Página &amp;P de &amp;N</oddFooter>
+    <oddFooter>MIPER-001 V3 | borrador | 2026-07-21 | Página &amp;P de &amp;N</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K3"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -2195,152 +1811,44 @@
     </row>
     <row r="3">
       <c r="A3" t="str" s="23">
-        <v>Recepción, almacenamiento y despacho</v>
+        <v>Operacion mina</v>
       </c>
       <c r="B3" t="str" s="23">
         <v>operacional</v>
       </c>
       <c r="C3" t="str" s="23">
-        <v>Operador de bodega</v>
+        <v>Operador</v>
       </c>
       <c r="D3" t="str" s="23">
-        <v>Recepcionar y almacenar materiales</v>
+        <v>Traslado interno</v>
       </c>
       <c r="E3" t="str" s="23">
         <v>Sí</v>
       </c>
       <c r="F3" t="str" s="23">
-        <v>Bodega central</v>
+        <v>Patio A</v>
       </c>
       <c r="G3" s="23">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H3" t="str" s="23">
-        <v>hombre: 2 | mujer: 2</v>
+        <v>hombre: 2 | mujer: 1</v>
       </c>
       <c r="I3" t="str" s="23">
-        <v>Gente: Personas expuestas durante la tarea | Equipos: Equipos móviles y herramientas | Materiales: Materiales almacenados | Ambiente: Superficie y condiciones del lugar | Detalle: Interacción observable durante la ejecución</v>
+        <v>Gente: Conductor fatigado | Equipos: Camioneta en maniobra | Detalle: Cruce sin demarcacion</v>
       </c>
       <c r="J3" t="str" s="23">
-        <v>A1 Caídas al mismo nivel | R1 Manipulación manual de cargas</v>
+        <v>I1 Atropello</v>
       </c>
       <c r="K3" t="str" s="23">
-        <v>Turno diurno</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str" s="24">
-        <v>Recepción, almacenamiento y despacho</v>
-      </c>
-      <c r="B4" t="str" s="24">
-        <v>operacional</v>
-      </c>
-      <c r="C4" t="str" s="24">
-        <v>Operador de bodega</v>
-      </c>
-      <c r="D4" t="str" s="24">
-        <v>Preparar pedidos para despacho</v>
-      </c>
-      <c r="E4" t="str" s="24">
-        <v>Sí</v>
-      </c>
-      <c r="F4" t="str" s="24">
-        <v>Zona de picking</v>
-      </c>
-      <c r="G4" s="24">
-        <v>3</v>
-      </c>
-      <c r="H4" t="str" s="24">
-        <v>hombre: 2 | mujer: 1</v>
-      </c>
-      <c r="I4" t="str" s="24">
-        <v>Gente: Personas expuestas durante la tarea | Equipos: Equipos móviles y herramientas | Materiales: Materiales almacenados | Ambiente: Superficie y condiciones del lugar | Detalle: Interacción observable durante la ejecución</v>
-      </c>
-      <c r="J4" t="str" s="24">
-        <v>B3 Cortes por herramientas | B2 Caída de objetos | P1 Exposición a ruido</v>
-      </c>
-      <c r="K4" t="str" s="24">
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str" s="23">
-        <v>Recepción, almacenamiento y despacho</v>
-      </c>
-      <c r="B5" t="str" s="23">
-        <v>operacional</v>
-      </c>
-      <c r="C5" t="str" s="23">
-        <v>Supervisor de operaciones</v>
-      </c>
-      <c r="D5" t="str" s="23">
-        <v>Supervisar operación y coordinar turnos</v>
-      </c>
-      <c r="E5" t="str" s="23">
-        <v>Sí</v>
-      </c>
-      <c r="F5" t="str" s="23">
-        <v>Bodega y oficina</v>
-      </c>
-      <c r="G5" s="23">
-        <v>2</v>
-      </c>
-      <c r="H5" t="str" s="23">
-        <v>hombre: 1 | mujer: 1</v>
-      </c>
-      <c r="I5" t="str" s="23">
-        <v>Gente: Personas expuestas durante la tarea | Equipos: Equipos móviles y herramientas | Materiales: Materiales almacenados | Ambiente: Superficie y condiciones del lugar | Detalle: Interacción observable durante la ejecución</v>
-      </c>
-      <c r="J5" t="str" s="23">
-        <v>D1 Carga de trabajo</v>
-      </c>
-      <c r="K5" t="str" s="23">
-        <v>Incluye recorridos</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str" s="24">
-        <v>Recepción, almacenamiento y despacho</v>
-      </c>
-      <c r="B6" t="str" s="24">
-        <v>operacional</v>
-      </c>
-      <c r="C6" t="str" s="24">
-        <v>Supervisor de operaciones</v>
-      </c>
-      <c r="D6" t="str" s="24">
-        <v>Gestionar contingencias operacionales</v>
-      </c>
-      <c r="E6" t="str" s="24">
-        <v>No</v>
-      </c>
-      <c r="F6" t="str" s="24">
-        <v>Instalación completa</v>
-      </c>
-      <c r="G6" s="24">
-        <v>2</v>
-      </c>
-      <c r="H6" t="str" s="24">
-        <v>hombre: 1 | mujer: 1</v>
-      </c>
-      <c r="I6" t="str" s="24">
-        <v>Gente: Personas expuestas durante la tarea | Equipos: Equipos móviles y herramientas | Materiales: Materiales almacenados | Ambiente: Superficie y condiciones del lugar | Detalle: Interacción observable durante la ejecución</v>
-      </c>
-      <c r="J6" t="str" s="24">
-        <v>F1 Contacto eléctrico directo</v>
-      </c>
-      <c r="K6" t="str" s="24">
-        <v>Según evento</v>
+        <v>Ruta principal</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:K6"/>
+  <autoFilter ref="A2:K3"/>
   <mergeCells count="1">
     <mergeCell ref="A1:K1"/>
   </mergeCells>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K6"/>
-  </ignoredErrors>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.45" header="0.15" footer="0.2"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
@@ -2352,7 +1860,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J3"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -2405,300 +1913,41 @@
     </row>
     <row r="3">
       <c r="A3" t="str" s="23">
-        <v>Recepción, almacenamiento y despacho</v>
+        <v>Operacion mina</v>
       </c>
       <c r="B3" t="str" s="23">
-        <v>Operador de bodega</v>
+        <v>Operador</v>
       </c>
       <c r="C3" t="str" s="23">
-        <v>Recepcionar y almacenar materiales</v>
+        <v>Traslado interno</v>
       </c>
       <c r="D3" t="str" s="23">
-        <v>A1</v>
+        <v>I1</v>
       </c>
       <c r="E3" t="str" s="23">
-        <v>Caídas al mismo nivel</v>
+        <v>Atropello</v>
       </c>
       <c r="F3" t="str" s="23">
         <v>Administrativo</v>
       </c>
       <c r="G3" t="str" s="23">
-        <v>Demarcar rutas y verificar orden y limpieza</v>
+        <v>Control de velocidad</v>
       </c>
       <c r="H3" t="str" s="23">
-        <v>Jefatura de operaciones</v>
+        <v>Juan Soto</v>
       </c>
       <c r="I3" t="str" s="23">
-        <v>2026-08-15</v>
+        <v>2026-07-20</v>
       </c>
       <c r="J3" t="str" s="25">
         <v>pendiente</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="str" s="24">
-        <v>Recepción, almacenamiento y despacho</v>
-      </c>
-      <c r="B4" t="str" s="24">
-        <v>Operador de bodega</v>
-      </c>
-      <c r="C4" t="str" s="24">
-        <v>Recepcionar y almacenar materiales</v>
-      </c>
-      <c r="D4" t="str" s="24">
-        <v>A1</v>
-      </c>
-      <c r="E4" t="str" s="24">
-        <v>Caídas al mismo nivel</v>
-      </c>
-      <c r="F4" t="str" s="24">
-        <v>Administrativo</v>
-      </c>
-      <c r="G4" t="str" s="24">
-        <v>Inspección diaria de superficies</v>
-      </c>
-      <c r="H4" t="str" s="24">
-        <v>Jefatura de operaciones</v>
-      </c>
-      <c r="I4" t="str" s="24">
-        <v>2026-08-15</v>
-      </c>
-      <c r="J4" t="str" s="26">
-        <v>implementado</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str" s="23">
-        <v>Recepción, almacenamiento y despacho</v>
-      </c>
-      <c r="B5" t="str" s="23">
-        <v>Operador de bodega</v>
-      </c>
-      <c r="C5" t="str" s="23">
-        <v>Preparar pedidos para despacho</v>
-      </c>
-      <c r="D5" t="str" s="23">
-        <v>B3</v>
-      </c>
-      <c r="E5" t="str" s="23">
-        <v>Cortes por herramientas</v>
-      </c>
-      <c r="F5" t="str" s="23">
-        <v>Administrativo</v>
-      </c>
-      <c r="G5" t="str" s="23">
-        <v>Usar cuchillos de seguridad y capacitar al personal</v>
-      </c>
-      <c r="H5" t="str" s="23">
-        <v>Jefatura de operaciones</v>
-      </c>
-      <c r="I5" t="str" s="23">
-        <v>2026-08-15</v>
-      </c>
-      <c r="J5" t="str" s="25">
-        <v>pendiente</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str" s="24">
-        <v>Recepción, almacenamiento y despacho</v>
-      </c>
-      <c r="B6" t="str" s="24">
-        <v>Operador de bodega</v>
-      </c>
-      <c r="C6" t="str" s="24">
-        <v>Preparar pedidos para despacho</v>
-      </c>
-      <c r="D6" t="str" s="24">
-        <v>B2</v>
-      </c>
-      <c r="E6" t="str" s="24">
-        <v>Caída de objetos</v>
-      </c>
-      <c r="F6" t="str" s="24">
-        <v>Administrativo</v>
-      </c>
-      <c r="G6" t="str" s="24">
-        <v>Reorganizar almacenamiento pesado</v>
-      </c>
-      <c r="H6" t="str" s="24">
-        <v>Jefatura de operaciones</v>
-      </c>
-      <c r="I6" t="str" s="24">
-        <v>2026-08-15</v>
-      </c>
-      <c r="J6" t="str" s="27">
-        <v>en_revision</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str" s="23">
-        <v>Recepción, almacenamiento y despacho</v>
-      </c>
-      <c r="B7" t="str" s="23">
-        <v>Operador de bodega</v>
-      </c>
-      <c r="C7" t="str" s="23">
-        <v>Preparar pedidos para despacho</v>
-      </c>
-      <c r="D7" t="str" s="23">
-        <v>B2</v>
-      </c>
-      <c r="E7" t="str" s="23">
-        <v>Caída de objetos</v>
-      </c>
-      <c r="F7" t="str" s="23">
-        <v>Administrativo</v>
-      </c>
-      <c r="G7" t="str" s="23">
-        <v>Instalar topes de retención</v>
-      </c>
-      <c r="H7" t="str" s="23">
-        <v>Jefatura de operaciones</v>
-      </c>
-      <c r="I7" t="str" s="23">
-        <v>2026-08-15</v>
-      </c>
-      <c r="J7" t="str" s="25">
-        <v>pendiente</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str" s="24">
-        <v>Recepción, almacenamiento y despacho</v>
-      </c>
-      <c r="B8" t="str" s="24">
-        <v>Supervisor de operaciones</v>
-      </c>
-      <c r="C8" t="str" s="24">
-        <v>Gestionar contingencias operacionales</v>
-      </c>
-      <c r="D8" t="str" s="24">
-        <v>F1</v>
-      </c>
-      <c r="E8" t="str" s="24">
-        <v>Contacto eléctrico directo</v>
-      </c>
-      <c r="F8" t="str" s="24">
-        <v>Administrativo</v>
-      </c>
-      <c r="G8" t="str" s="24">
-        <v>Retirar equipo defectuoso y bloquear energías</v>
-      </c>
-      <c r="H8" t="str" s="24">
-        <v>Jefatura de operaciones</v>
-      </c>
-      <c r="I8" t="str" s="24">
-        <v>2026-08-15</v>
-      </c>
-      <c r="J8" t="str" s="25">
-        <v>pendiente</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str" s="23">
-        <v>Recepción, almacenamiento y despacho</v>
-      </c>
-      <c r="B9" t="str" s="23">
-        <v>Operador de bodega</v>
-      </c>
-      <c r="C9" t="str" s="23">
-        <v>Preparar pedidos para despacho</v>
-      </c>
-      <c r="D9" t="str" s="23">
-        <v>P1</v>
-      </c>
-      <c r="E9" t="str" s="23">
-        <v>Exposición a ruido</v>
-      </c>
-      <c r="F9" t="str" s="23">
-        <v>Administrativo</v>
-      </c>
-      <c r="G9" t="str" s="23">
-        <v>Implementar programa de conservación auditiva</v>
-      </c>
-      <c r="H9" t="str" s="23">
-        <v>Jefatura de operaciones</v>
-      </c>
-      <c r="I9" t="str" s="23">
-        <v>2026-08-15</v>
-      </c>
-      <c r="J9" t="str" s="25">
-        <v>pendiente</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str" s="24">
-        <v>Recepción, almacenamiento y despacho</v>
-      </c>
-      <c r="B10" t="str" s="24">
-        <v>Supervisor de operaciones</v>
-      </c>
-      <c r="C10" t="str" s="24">
-        <v>Supervisar operación y coordinar turnos</v>
-      </c>
-      <c r="D10" t="str" s="24">
-        <v>D1</v>
-      </c>
-      <c r="E10" t="str" s="24">
-        <v>Carga de trabajo</v>
-      </c>
-      <c r="F10" t="str" s="24">
-        <v>Administrativo</v>
-      </c>
-      <c r="G10" t="str" s="24">
-        <v>Revisar distribución de carga y pausas</v>
-      </c>
-      <c r="H10" t="str" s="24">
-        <v>Jefatura de operaciones</v>
-      </c>
-      <c r="I10" t="str" s="24">
-        <v>2026-08-15</v>
-      </c>
-      <c r="J10" t="str" s="25">
-        <v>pendiente</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str" s="23">
-        <v>Recepción, almacenamiento y despacho</v>
-      </c>
-      <c r="B11" t="str" s="23">
-        <v>Operador de bodega</v>
-      </c>
-      <c r="C11" t="str" s="23">
-        <v>Recepcionar y almacenar materiales</v>
-      </c>
-      <c r="D11" t="str" s="23">
-        <v>R1</v>
-      </c>
-      <c r="E11" t="str" s="23">
-        <v>Manipulación manual de cargas</v>
-      </c>
-      <c r="F11" t="str" s="23">
-        <v>Administrativo</v>
-      </c>
-      <c r="G11" t="str" s="23">
-        <v>Incorporar ayuda mecánica para cargas</v>
-      </c>
-      <c r="H11" t="str" s="23">
-        <v>Jefatura de operaciones</v>
-      </c>
-      <c r="I11" t="str" s="23">
-        <v>2026-08-15</v>
-      </c>
-      <c r="J11" t="str" s="25">
-        <v>pendiente</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A2:J11"/>
+  <autoFilter ref="A2:J3"/>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J11"/>
-  </ignoredErrors>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.45" header="0.15" footer="0.2"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
@@ -2710,7 +1959,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G3"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -2751,16 +2000,16 @@
     </row>
     <row r="3">
       <c r="A3" t="str" s="23">
-        <v>A1</v>
+        <v>I1</v>
       </c>
       <c r="B3" t="str" s="23">
-        <v>Caída de personas</v>
+        <v>Contacto con / en Vehículos en movimiento</v>
       </c>
       <c r="C3" t="str" s="23">
-        <v>Caídas al mismo nivel</v>
+        <v>Atropellos o golpes con vehículos</v>
       </c>
       <c r="D3" t="str" s="23">
-        <v>Caída que se produce en el mismo plano de sustentación, por ejemplo: caídas en lugares de tránsito o superficies de trabajo, caídas sobre o contra objetos.</v>
+        <v>Impacto entre un peatón y un vehículo en movimiento.</v>
       </c>
       <c r="E3" t="str" s="23">
         <v>seguridad</v>
@@ -2772,153 +2021,11 @@
         <v/>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="str" s="24">
-        <v>B2</v>
-      </c>
-      <c r="B4" t="str" s="24">
-        <v>Contacto con objetos</v>
-      </c>
-      <c r="C4" t="str" s="24">
-        <v>Caída de objetos</v>
-      </c>
-      <c r="D4" t="str" s="24">
-        <v>Caída de elementos que golpean al cuerpo, por ejemplo, materiales, herramientas, estructuras, etc.</v>
-      </c>
-      <c r="E4" t="str" s="24">
-        <v>seguridad</v>
-      </c>
-      <c r="F4" t="str" s="24">
-        <v>vep_isp</v>
-      </c>
-      <c r="G4" t="str" s="24">
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str" s="23">
-        <v>B3</v>
-      </c>
-      <c r="B5" t="str" s="23">
-        <v>Contacto con objetos</v>
-      </c>
-      <c r="C5" t="str" s="23">
-        <v>Cortes por objetos / herramientas corto-punzantes</v>
-      </c>
-      <c r="D5" t="str" s="23">
-        <v>Cortes y/o punzaciones generadas en parte del cuerpo debido al contacto de éste con objetos cortantes, punzantes y/o abrasivos.</v>
-      </c>
-      <c r="E5" t="str" s="23">
-        <v>seguridad</v>
-      </c>
-      <c r="F5" t="str" s="23">
-        <v>vep_isp</v>
-      </c>
-      <c r="G5" t="str" s="23">
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str" s="24">
-        <v>F1</v>
-      </c>
-      <c r="B6" t="str" s="24">
-        <v>Contacto con energía eléctrica</v>
-      </c>
-      <c r="C6" t="str" s="24">
-        <v>Contactos eléctricos directos baja tensión</v>
-      </c>
-      <c r="D6" t="str" s="24">
-        <v>Es todo contacto directo de las personas con partes activas en tensión (trabajando con tensiones menores a 1000 volts).</v>
-      </c>
-      <c r="E6" t="str" s="24">
-        <v>seguridad</v>
-      </c>
-      <c r="F6" t="str" s="24">
-        <v>vep_isp</v>
-      </c>
-      <c r="G6" t="str" s="24">
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str" s="23">
-        <v>P1</v>
-      </c>
-      <c r="B7" t="str" s="23">
-        <v>Exposición a agentes físicos</v>
-      </c>
-      <c r="C7" t="str" s="23">
-        <v>Exposición a ruido</v>
-      </c>
-      <c r="D7" t="str" s="23">
-        <v>Permanencia en un ambiente de trabajo con presencia continua de altos niveles de presión sonora (en forma estable o fluctuante), con la potencialidad de alterar el órgano de la audición.</v>
-      </c>
-      <c r="E7" t="str" s="23">
-        <v>higienico</v>
-      </c>
-      <c r="F7" t="str" s="23">
-        <v>evaluacion_especifica</v>
-      </c>
-      <c r="G7" t="str" s="23">
-        <v>Protocolo de Exposición Ocupacional a Ruido (PREXOR)</v>
-      </c>
-    </row>
-    <row r="8" xml:space="preserve">
-      <c r="A8" t="str" s="24">
-        <v>R1</v>
-      </c>
-      <c r="B8" t="str" s="24">
-        <v>Manejo o Manipulación Manual de Carga (MMC) o personas /Pacientes (MMP)</v>
-      </c>
-      <c r="C8" t="str" s="24">
-        <v>Sobrecarga física debido a la manipulación manual de cargas</v>
-      </c>
-      <c r="D8" t="str" xml:space="preserve" s="24">
-        <v xml:space="preserve">Trabajos en donde se deban levantar, descender o transportar manualmente objetos de más de 3 kilos.
-Trabajos en donde se deban empujar o arrastrar objetos utilizando 1 o 2 manos.</v>
-      </c>
-      <c r="E8" t="str" s="24">
-        <v>musculoesqueletico</v>
-      </c>
-      <c r="F8" t="str" s="24">
-        <v>evaluacion_especifica</v>
-      </c>
-      <c r="G8" t="str" s="24">
-        <v>Guía técnica para la evaluación y control de riesgos asociados al manejo o manipulación manual de carga</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str" s="23">
-        <v>D1</v>
-      </c>
-      <c r="B9" t="str" s="23">
-        <v>Riesgos psicosociales laborales</v>
-      </c>
-      <c r="C9" t="str" s="23">
-        <v>1. Dimensión carga de trabajo (CT).</v>
-      </c>
-      <c r="D9" t="str" s="23">
-        <v>La carga de trabajo son las exigencias que se le hacen a los trabajadores y trabajadoras para que cumplan con un determinado objetivo o tarea en un tiempo acotado o limitado. Es decir, en la carga de trabajo existe una relación entre la cantidad de tareas y el tiempo en que se deben realizar, que puede ser desde minutos hasta semanas o más.</v>
-      </c>
-      <c r="E9" t="str" s="23">
-        <v>psicosocial</v>
-      </c>
-      <c r="F9" t="str" s="23">
-        <v>evaluacion_especifica</v>
-      </c>
-      <c r="G9" t="str" s="23">
-        <v>Protocolo de vigilancia de riesgos psicosociales en el trabajo</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A2:G9"/>
+  <autoFilter ref="A2:G3"/>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G9"/>
-  </ignoredErrors>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.45" header="0.15" footer="0.2"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
@@ -2930,7 +2037,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G7"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -2951,13 +2058,13 @@
         <v>Código</v>
       </c>
       <c r="B2" t="str" s="5">
-        <v>MIPER-PRUEBA-001</v>
+        <v>MIPER-001</v>
       </c>
       <c r="C2" t="str" s="4">
         <v>Versión</v>
       </c>
       <c r="D2" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E2" t="str" s="4">
         <v>Estado</v>
@@ -2971,13 +2078,13 @@
         <v>Versión anterior</v>
       </c>
       <c r="B3" t="str" s="5">
-        <v>No informado</v>
+        <v>MIPER-001-V2</v>
       </c>
       <c r="C3" t="str" s="4">
         <v>Fecha descarga</v>
       </c>
       <c r="D3" t="str" s="5">
-        <v>2026-07-20</v>
+        <v>2026-07-21</v>
       </c>
       <c r="E3" t="str" s="4">
         <v>Nota legacy</v>
@@ -2991,7 +2098,7 @@
         <v>Elaborado por</v>
       </c>
       <c r="B4" t="str" s="5">
-        <v>Diana Marín · Prevencionista de riesgos</v>
+        <v>Ana Perez</v>
       </c>
       <c r="C4" t="str" s="4">
         <v>Revisado por</v>
@@ -3031,16 +2138,16 @@
     </row>
     <row r="7">
       <c r="A7" t="str" s="23">
-        <v>i1</v>
+        <v>i-1</v>
       </c>
       <c r="B7" t="str" s="23">
-        <v>t1</v>
+        <v>t-1</v>
       </c>
       <c r="C7" t="str" s="23">
         <v>vep_isp</v>
       </c>
       <c r="D7" t="str" s="23">
-        <v>Confirmado durante levantamiento ISP</v>
+        <v>Mapeo por exposicion</v>
       </c>
       <c r="E7" t="str" s="23">
         <v>vep</v>
@@ -3049,178 +2156,14 @@
         <v/>
       </c>
       <c r="G7" t="str" s="23">
-        <v>Responsable: Jefatura de operaciones | Protocolo: No informado</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str" s="24">
-        <v>i2</v>
-      </c>
-      <c r="B8" t="str" s="24">
-        <v>t1</v>
-      </c>
-      <c r="C8" t="str" s="24">
-        <v>vep_isp</v>
-      </c>
-      <c r="D8" t="str" s="24">
-        <v>Confirmado durante levantamiento ISP</v>
-      </c>
-      <c r="E8" t="str" s="24">
-        <v>vep</v>
-      </c>
-      <c r="F8" t="str" s="24">
-        <v/>
-      </c>
-      <c r="G8" t="str" s="24">
-        <v>Responsable: Jefatura de operaciones | Protocolo: No informado</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str" s="23">
-        <v>i3</v>
-      </c>
-      <c r="B9" t="str" s="23">
-        <v>t2</v>
-      </c>
-      <c r="C9" t="str" s="23">
-        <v>vep_isp</v>
-      </c>
-      <c r="D9" t="str" s="23">
-        <v>Confirmado durante levantamiento ISP</v>
-      </c>
-      <c r="E9" t="str" s="23">
-        <v>vep</v>
-      </c>
-      <c r="F9" t="str" s="23">
-        <v/>
-      </c>
-      <c r="G9" t="str" s="23">
-        <v>Responsable: Jefatura de operaciones | Protocolo: No informado</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str" s="24">
-        <v>i4</v>
-      </c>
-      <c r="B10" t="str" s="24">
-        <v>t2</v>
-      </c>
-      <c r="C10" t="str" s="24">
-        <v>vep_isp</v>
-      </c>
-      <c r="D10" t="str" s="24">
-        <v>Confirmado durante levantamiento ISP</v>
-      </c>
-      <c r="E10" t="str" s="24">
-        <v>vep</v>
-      </c>
-      <c r="F10" t="str" s="24">
-        <v/>
-      </c>
-      <c r="G10" t="str" s="24">
-        <v>Responsable: Jefatura de operaciones | Protocolo: No informado</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str" s="23">
-        <v>i5</v>
-      </c>
-      <c r="B11" t="str" s="23">
-        <v>t4</v>
-      </c>
-      <c r="C11" t="str" s="23">
-        <v>vep_isp</v>
-      </c>
-      <c r="D11" t="str" s="23">
-        <v>Confirmado durante levantamiento ISP</v>
-      </c>
-      <c r="E11" t="str" s="23">
-        <v>vep</v>
-      </c>
-      <c r="F11" t="str" s="23">
-        <v/>
-      </c>
-      <c r="G11" t="str" s="23">
-        <v>Responsable: Jefatura de operaciones | Protocolo: No informado</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str" s="24">
-        <v>i6</v>
-      </c>
-      <c r="B12" t="str" s="24">
-        <v>t2</v>
-      </c>
-      <c r="C12" t="str" s="24">
-        <v>evaluacion_especifica</v>
-      </c>
-      <c r="D12" t="str" s="24">
-        <v>Confirmado durante levantamiento ISP</v>
-      </c>
-      <c r="E12" t="str" s="24">
-        <v>evaluado</v>
-      </c>
-      <c r="F12" t="str" s="24">
-        <v>Medición higiénica programada</v>
-      </c>
-      <c r="G12" t="str" s="24">
-        <v>Responsable: Jefatura de operaciones | Protocolo: PREXOR</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str" s="23">
-        <v>i7</v>
-      </c>
-      <c r="B13" t="str" s="23">
-        <v>t3</v>
-      </c>
-      <c r="C13" t="str" s="23">
-        <v>evaluacion_especifica</v>
-      </c>
-      <c r="D13" t="str" s="23">
-        <v>Confirmado durante levantamiento ISP</v>
-      </c>
-      <c r="E13" t="str" s="23">
-        <v>evaluado</v>
-      </c>
-      <c r="F13" t="str" s="23">
-        <v>Resultado por unidad</v>
-      </c>
-      <c r="G13" t="str" s="23">
-        <v>Responsable: Jefatura de operaciones | Protocolo: CEAL-SM/SUSESO</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str" s="24">
-        <v>i8</v>
-      </c>
-      <c r="B14" t="str" s="24">
-        <v>t1</v>
-      </c>
-      <c r="C14" t="str" s="24">
-        <v>evaluacion_especifica</v>
-      </c>
-      <c r="D14" t="str" s="24">
-        <v>Confirmado durante levantamiento ISP</v>
-      </c>
-      <c r="E14" t="str" s="24">
-        <v>evaluado</v>
-      </c>
-      <c r="F14" t="str" s="24">
-        <v>Evaluación inicial</v>
-      </c>
-      <c r="G14" t="str" s="24">
-        <v>Responsable: Jefatura de operaciones | Protocolo: MMC</v>
+        <v>Responsable: Juan Soto | Protocolo: No informado</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:G14"/>
+  <autoFilter ref="A6:G7"/>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G14"/>
-  </ignoredErrors>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.45" header="0.15" footer="0.2"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>